<commit_message>
feat(proposal): add ALUMINIUM_WEIGHT and BLOCKS_WEIGHT to proposal template
Compute total aluminium weight (angle + rail profiles, excl. depreciation)
and total blocks weight (block_50x24x15) from the effective BOM and inject
into the corresponding template placeholder cells. Also exclude
depreciation_waste from the BOM header aluminium weight stat in the FE.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BE/mgp-service/app/templates/proposal_template.xlsx
+++ b/BE/mgp-service/app/templates/proposal_template.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10503"/>
   <workbookPr filterPrivacy="1" codeName="ThisWorkbook"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7C7193AD-03D7-9A42-A8AB-118A7FCD0A3C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B5A6DDC3-89D5-364A-ADEE-326CDD5EB49F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="38400" windowHeight="19720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="19720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="pricing" sheetId="2" r:id="rId1"/>
@@ -19,8 +19,8 @@
     <definedName name="CLIENT_NAME">[1]ראשי!#REF!</definedName>
     <definedName name="OFFER_DATE">[1]ראשי!#REF!</definedName>
     <definedName name="OFFER_VALID_TO">[1]ראשי!#REF!</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">pricing!$A$1:$I$28</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">quantities!$A$1:$L$17</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">pricing!$A$1:$I$30</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">quantities!$A$1:$L$19</definedName>
     <definedName name="prOJECT_NAME">[1]ראשי!#REF!</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="45">
   <si>
     <t>שורה</t>
   </si>
@@ -172,6 +172,18 @@
   </si>
   <si>
     <t>QTY_TABLE_DATA_ROW</t>
+  </si>
+  <si>
+    <t>משקל אבנים (ק"ג)</t>
+  </si>
+  <si>
+    <t>משקל אלומיניום (ק"ג)</t>
+  </si>
+  <si>
+    <t>BLOCKS_WEIGHT</t>
+  </si>
+  <si>
+    <t>ALUMINIUM_WEIGHT</t>
   </si>
 </sst>
 </file>
@@ -329,7 +341,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="4">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -378,12 +390,36 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="56">
+  <cellXfs count="61">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -515,19 +551,43 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="18" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" readingOrder="2"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="12" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="18" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="12" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="18" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" readingOrder="2"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" readingOrder="2"/>
     </xf>
@@ -536,15 +596,6 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1" readingOrder="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" readingOrder="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -565,25 +616,8 @@
         <vertAlign val="baseline"/>
         <sz val="12"/>
         <color rgb="FF000000"/>
-        <name val="Heebo"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <name val="Heebo"/>
+        <name val="Calibri"/>
+        <family val="2"/>
         <scheme val="none"/>
       </font>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -620,7 +654,8 @@
         <vertAlign val="baseline"/>
         <sz val="12"/>
         <color rgb="FF000000"/>
-        <name val="Heebo"/>
+        <name val="Calibri"/>
+        <family val="2"/>
         <scheme val="none"/>
       </font>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -657,10 +692,10 @@
         <vertAlign val="baseline"/>
         <sz val="12"/>
         <color rgb="FF000000"/>
-        <name val="Heebo"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="4" formatCode="#,##0.00"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
@@ -695,12 +730,71 @@
         <vertAlign val="baseline"/>
         <sz val="12"/>
         <color rgb="FF000000"/>
-        <name val="Heebo"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <name val="Calibri"/>
+        <family val="2"/>
         <scheme val="none"/>
       </font>
       <numFmt numFmtId="4" formatCode="#,##0.00"/>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="4" formatCode="#,##0.00"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
         <left style="thin">
           <color indexed="64"/>
         </left>
@@ -713,6 +807,12 @@
         <bottom style="thin">
           <color indexed="64"/>
         </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
       </border>
     </dxf>
     <dxf>
@@ -784,7 +884,6 @@
         <strike val="0"/>
         <outline val="0"/>
         <shadow val="0"/>
-        <u val="none"/>
         <vertAlign val="baseline"/>
         <sz val="12"/>
         <name val="Heebo"/>
@@ -811,7 +910,6 @@
         <strike val="0"/>
         <outline val="0"/>
         <shadow val="0"/>
-        <u val="none"/>
         <vertAlign val="baseline"/>
         <sz val="12"/>
         <name val="Heebo"/>
@@ -837,7 +935,6 @@
         <strike val="0"/>
         <outline val="0"/>
         <shadow val="0"/>
-        <u val="none"/>
         <vertAlign val="baseline"/>
         <sz val="12"/>
         <name val="Heebo"/>
@@ -928,7 +1025,6 @@
         <strike val="0"/>
         <outline val="0"/>
         <shadow val="0"/>
-        <u val="none"/>
         <vertAlign val="baseline"/>
         <sz val="12"/>
         <name val="Heebo"/>
@@ -1004,7 +1100,8 @@
         <vertAlign val="baseline"/>
         <sz val="12"/>
         <color rgb="FF000000"/>
-        <name val="Heebo"/>
+        <name val="Calibri"/>
+        <family val="2"/>
         <scheme val="none"/>
       </font>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -1029,8 +1126,9 @@
         <vertAlign val="baseline"/>
         <sz val="12"/>
         <color theme="0"/>
-        <name val="Heebo"/>
-        <scheme val="none"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
       </font>
       <fill>
         <patternFill patternType="solid">
@@ -1063,8 +1161,25 @@
         <vertAlign val="baseline"/>
         <sz val="12"/>
         <color rgb="FF000000"/>
-        <name val="Calibri"/>
-        <family val="2"/>
+        <name val="Heebo"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <name val="Heebo"/>
         <scheme val="none"/>
       </font>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -1101,8 +1216,7 @@
         <vertAlign val="baseline"/>
         <sz val="12"/>
         <color rgb="FF000000"/>
-        <name val="Calibri"/>
-        <family val="2"/>
+        <name val="Heebo"/>
         <scheme val="none"/>
       </font>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -1139,10 +1253,10 @@
         <vertAlign val="baseline"/>
         <sz val="12"/>
         <color rgb="FF000000"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
+        <name val="Heebo"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="4" formatCode="#,##0.00"/>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
@@ -1177,71 +1291,12 @@
         <vertAlign val="baseline"/>
         <sz val="12"/>
         <color rgb="FF000000"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <name val="Calibri"/>
-        <family val="2"/>
+        <name val="Heebo"/>
         <scheme val="none"/>
       </font>
       <numFmt numFmtId="4" formatCode="#,##0.00"/>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="4" formatCode="#,##0.00"/>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
+      <border diagonalUp="0" diagonalDown="0" outline="0">
         <left style="thin">
           <color indexed="64"/>
         </left>
@@ -1254,12 +1309,6 @@
         <bottom style="thin">
           <color indexed="64"/>
         </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
       </border>
     </dxf>
     <dxf>
@@ -1331,6 +1380,7 @@
         <strike val="0"/>
         <outline val="0"/>
         <shadow val="0"/>
+        <u val="none"/>
         <vertAlign val="baseline"/>
         <sz val="12"/>
         <name val="Heebo"/>
@@ -1357,6 +1407,7 @@
         <strike val="0"/>
         <outline val="0"/>
         <shadow val="0"/>
+        <u val="none"/>
         <vertAlign val="baseline"/>
         <sz val="12"/>
         <name val="Heebo"/>
@@ -1382,6 +1433,7 @@
         <strike val="0"/>
         <outline val="0"/>
         <shadow val="0"/>
+        <u val="none"/>
         <vertAlign val="baseline"/>
         <sz val="12"/>
         <name val="Heebo"/>
@@ -1472,6 +1524,7 @@
         <strike val="0"/>
         <outline val="0"/>
         <shadow val="0"/>
+        <u val="none"/>
         <vertAlign val="baseline"/>
         <sz val="12"/>
         <name val="Heebo"/>
@@ -1547,8 +1600,7 @@
         <vertAlign val="baseline"/>
         <sz val="12"/>
         <color rgb="FF000000"/>
-        <name val="Calibri"/>
-        <family val="2"/>
+        <name val="Heebo"/>
         <scheme val="none"/>
       </font>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -1573,9 +1625,8 @@
         <vertAlign val="baseline"/>
         <sz val="12"/>
         <color theme="0"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
+        <name val="Heebo"/>
+        <scheme val="none"/>
       </font>
       <fill>
         <patternFill patternType="solid">
@@ -1632,48 +1683,48 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{5ACB1EC1-21C6-AF40-A140-308C9117B91F}" name="pricing_table25" displayName="pricing_table25" ref="B10:N11" totalsRowShown="0" headerRowDxfId="45" dataDxfId="43" totalsRowDxfId="41" headerRowBorderDxfId="44" tableBorderDxfId="42" totalsRowBorderDxfId="40">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{5ACB1EC1-21C6-AF40-A140-308C9117B91F}" name="pricing_table25" displayName="pricing_table25" ref="B10:N11" totalsRowShown="0" headerRowDxfId="23" dataDxfId="21" totalsRowDxfId="19" headerRowBorderDxfId="22" tableBorderDxfId="20" totalsRowBorderDxfId="18">
   <autoFilter ref="B10:N11" xr:uid="{A700047D-2A12-4A24-87A3-5C54C0CD36D6}"/>
   <tableColumns count="13">
-    <tableColumn id="1" xr3:uid="{9715C0F5-6C58-0C48-A92D-3904FFEE1286}" name="שורה" dataDxfId="39"/>
-    <tableColumn id="2" xr3:uid="{E71665ED-EE05-B544-8402-B3336F34DA2C}" name="מיקום בגג" dataDxfId="38"/>
-    <tableColumn id="3" xr3:uid="{58C96AFC-B01E-D446-8E2A-ACF7B2497559}" name="תאור מוצר" dataDxfId="37"/>
-    <tableColumn id="4" xr3:uid="{D9DC81BB-9F60-0047-86B9-14278D4E2EE7}" name="אורך" dataDxfId="36"/>
-    <tableColumn id="5" xr3:uid="{B9B74024-7469-A149-9639-A328A6F77916}" name="כמות" dataDxfId="35"/>
-    <tableColumn id="6" xr3:uid="{0FF2A4DA-EE5D-564C-892E-1BAF5895A4E7}" name="כמות: ק&quot;ג\יחידות" dataDxfId="34"/>
-    <tableColumn id="7" xr3:uid="{D3D78E52-A52E-C949-9ABD-03AD0269F0BF}" name="מחיר ליחידה (₪)" dataDxfId="33"/>
-    <tableColumn id="8" xr3:uid="{E1EB6162-FB78-1D4F-9435-2CE9366E3552}" name="סה&quot;כ מחיר (₪)" dataDxfId="32">
+    <tableColumn id="1" xr3:uid="{9715C0F5-6C58-0C48-A92D-3904FFEE1286}" name="שורה" dataDxfId="17"/>
+    <tableColumn id="2" xr3:uid="{E71665ED-EE05-B544-8402-B3336F34DA2C}" name="מיקום בגג" dataDxfId="16"/>
+    <tableColumn id="3" xr3:uid="{58C96AFC-B01E-D446-8E2A-ACF7B2497559}" name="תאור מוצר" dataDxfId="15"/>
+    <tableColumn id="4" xr3:uid="{D9DC81BB-9F60-0047-86B9-14278D4E2EE7}" name="אורך" dataDxfId="14"/>
+    <tableColumn id="5" xr3:uid="{B9B74024-7469-A149-9639-A328A6F77916}" name="כמות" dataDxfId="13"/>
+    <tableColumn id="6" xr3:uid="{0FF2A4DA-EE5D-564C-892E-1BAF5895A4E7}" name="כמות: ק&quot;ג\יחידות" dataDxfId="12"/>
+    <tableColumn id="7" xr3:uid="{D3D78E52-A52E-C949-9ABD-03AD0269F0BF}" name="מחיר ליחידה (₪)" dataDxfId="11"/>
+    <tableColumn id="8" xr3:uid="{E1EB6162-FB78-1D4F-9435-2CE9366E3552}" name="סה&quot;כ מחיר (₪)" dataDxfId="10">
       <calculatedColumnFormula>pricing_table25[[#This Row],[מחיר ליחידה (₪)]]*pricing_table25[[#This Row],[כמות: ק"ג\יחידות]]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{EAED02B8-7E3B-9B47-8C95-FD7B3D6B7DA0}" name="*כמות פחת" dataDxfId="31" totalsRowDxfId="30"/>
-    <tableColumn id="10" xr3:uid="{8DD3D515-E5F7-3F44-AEEC-EBD82CE3FE68}" name="סה&quot;כ מחיר כולל פחת (₪)" dataDxfId="29" totalsRowDxfId="28"/>
-    <tableColumn id="11" xr3:uid="{B17131E0-AD15-314F-8745-C01B5B56C8B5}" name="*משקל בק&quot;ג" dataDxfId="27" totalsRowDxfId="26"/>
-    <tableColumn id="12" xr3:uid="{8383AEF5-4B81-5944-B8C1-7A02610AD799}" name="&gt;% Discount - Construction" dataDxfId="25" totalsRowDxfId="24"/>
-    <tableColumn id="13" xr3:uid="{A6FF8C60-F61C-014D-BE3D-D97E0E91917D}" name="*סה&quot;כ מחיר כולל פחת אחרי הנחה (₪)" dataDxfId="23" totalsRowDxfId="22"/>
+    <tableColumn id="9" xr3:uid="{EAED02B8-7E3B-9B47-8C95-FD7B3D6B7DA0}" name="*כמות פחת" dataDxfId="9" totalsRowDxfId="8"/>
+    <tableColumn id="10" xr3:uid="{8DD3D515-E5F7-3F44-AEEC-EBD82CE3FE68}" name="סה&quot;כ מחיר כולל פחת (₪)" dataDxfId="7" totalsRowDxfId="6"/>
+    <tableColumn id="11" xr3:uid="{B17131E0-AD15-314F-8745-C01B5B56C8B5}" name="*משקל בק&quot;ג" dataDxfId="5" totalsRowDxfId="4"/>
+    <tableColumn id="12" xr3:uid="{8383AEF5-4B81-5944-B8C1-7A02610AD799}" name="&gt;% Discount - Construction" dataDxfId="3" totalsRowDxfId="2"/>
+    <tableColumn id="13" xr3:uid="{A6FF8C60-F61C-014D-BE3D-D97E0E91917D}" name="*סה&quot;כ מחיר כולל פחת אחרי הנחה (₪)" dataDxfId="1" totalsRowDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium15" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{53B791F9-974C-2D45-9198-4628741EC180}" name="pricing_table34" displayName="pricing_table34" ref="B10:N11" totalsRowShown="0" headerRowDxfId="21" dataDxfId="19" totalsRowDxfId="17" headerRowBorderDxfId="20" tableBorderDxfId="18" totalsRowBorderDxfId="16">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{53B791F9-974C-2D45-9198-4628741EC180}" name="pricing_table34" displayName="pricing_table34" ref="B10:N11" totalsRowShown="0" headerRowDxfId="45" dataDxfId="43" totalsRowDxfId="41" headerRowBorderDxfId="44" tableBorderDxfId="42" totalsRowBorderDxfId="40">
   <autoFilter ref="B10:N11" xr:uid="{A700047D-2A12-4A24-87A3-5C54C0CD36D6}"/>
   <tableColumns count="13">
-    <tableColumn id="1" xr3:uid="{C9E84F90-D937-9240-8769-8F47365B79B5}" name="שורה" dataDxfId="15"/>
-    <tableColumn id="2" xr3:uid="{584DEAFB-76D6-C647-A742-316CAAE5BC89}" name="מיקום בגג" dataDxfId="14"/>
-    <tableColumn id="3" xr3:uid="{199A858B-5154-3C42-B14B-B655372B7E72}" name="תאור מוצר" dataDxfId="13"/>
-    <tableColumn id="4" xr3:uid="{044A01A8-0D84-EB4C-A2F1-510AF1F79EC1}" name="אורך" dataDxfId="12"/>
-    <tableColumn id="5" xr3:uid="{23494D31-1003-EC4A-B3E4-56115FE1DC9B}" name="כמות" dataDxfId="11"/>
-    <tableColumn id="6" xr3:uid="{C3ADA01B-011E-AF49-B8EF-BF51E4952D25}" name="כמות: ק&quot;ג\יחידות" dataDxfId="10"/>
-    <tableColumn id="7" xr3:uid="{A4F8123E-37EB-2544-80EC-813AFA9298EC}" name="מחיר ליחידה (₪)" dataDxfId="9"/>
-    <tableColumn id="8" xr3:uid="{891F3848-661F-3446-A7E0-95642AC543B8}" name="סה&quot;כ מחיר (₪)" dataDxfId="8">
+    <tableColumn id="1" xr3:uid="{C9E84F90-D937-9240-8769-8F47365B79B5}" name="שורה" dataDxfId="39"/>
+    <tableColumn id="2" xr3:uid="{584DEAFB-76D6-C647-A742-316CAAE5BC89}" name="מיקום בגג" dataDxfId="38"/>
+    <tableColumn id="3" xr3:uid="{199A858B-5154-3C42-B14B-B655372B7E72}" name="תאור מוצר" dataDxfId="37"/>
+    <tableColumn id="4" xr3:uid="{044A01A8-0D84-EB4C-A2F1-510AF1F79EC1}" name="אורך" dataDxfId="36"/>
+    <tableColumn id="5" xr3:uid="{23494D31-1003-EC4A-B3E4-56115FE1DC9B}" name="כמות" dataDxfId="35"/>
+    <tableColumn id="6" xr3:uid="{C3ADA01B-011E-AF49-B8EF-BF51E4952D25}" name="כמות: ק&quot;ג\יחידות" dataDxfId="34"/>
+    <tableColumn id="7" xr3:uid="{A4F8123E-37EB-2544-80EC-813AFA9298EC}" name="מחיר ליחידה (₪)" dataDxfId="33"/>
+    <tableColumn id="8" xr3:uid="{891F3848-661F-3446-A7E0-95642AC543B8}" name="סה&quot;כ מחיר (₪)" dataDxfId="32">
       <calculatedColumnFormula>pricing_table34[[#This Row],[מחיר ליחידה (₪)]]*pricing_table34[[#This Row],[כמות: ק"ג\יחידות]]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{A50A1AEB-0486-8F4C-A4F6-1B417D72DF83}" name="*כמות פחת" dataDxfId="7" totalsRowDxfId="6"/>
-    <tableColumn id="10" xr3:uid="{3B89E727-3B11-4A40-B717-5C248FA24D57}" name="סה&quot;כ מחיר כולל פחת (₪)" dataDxfId="5" totalsRowDxfId="4"/>
-    <tableColumn id="11" xr3:uid="{981756E0-FF9F-014E-A803-EA2D248E751E}" name="*משקל בק&quot;ג" dataDxfId="3" totalsRowDxfId="2"/>
-    <tableColumn id="12" xr3:uid="{DAD5CC53-679B-024A-96B0-9223C3E03988}" name="&gt;% Discount - Construction" dataDxfId="1"/>
-    <tableColumn id="13" xr3:uid="{7498AF7D-E4AF-4D4F-A51C-BC365E54108A}" name="*סה&quot;כ מחיר כולל פחת אחרי הנחה (₪)" dataDxfId="0"/>
+    <tableColumn id="9" xr3:uid="{A50A1AEB-0486-8F4C-A4F6-1B417D72DF83}" name="*כמות פחת" dataDxfId="31" totalsRowDxfId="30"/>
+    <tableColumn id="10" xr3:uid="{3B89E727-3B11-4A40-B717-5C248FA24D57}" name="סה&quot;כ מחיר כולל פחת (₪)" dataDxfId="29" totalsRowDxfId="28"/>
+    <tableColumn id="11" xr3:uid="{981756E0-FF9F-014E-A803-EA2D248E751E}" name="*משקל בק&quot;ג" dataDxfId="27" totalsRowDxfId="26"/>
+    <tableColumn id="12" xr3:uid="{DAD5CC53-679B-024A-96B0-9223C3E03988}" name="&gt;% Discount - Construction" dataDxfId="25"/>
+    <tableColumn id="13" xr3:uid="{7498AF7D-E4AF-4D4F-A51C-BC365E54108A}" name="*סה&quot;כ מחיר כולל פחת אחרי הנחה (₪)" dataDxfId="24"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium15" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2004,7 +2055,7 @@
   <sheetPr codeName="Sheet5">
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:T35"/>
+  <dimension ref="A1:T37"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.1640625" defaultRowHeight="20" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="2.5" style="3" customWidth="1"/>
@@ -2013,8 +2064,7 @@
     <col min="4" max="4" width="26.1640625" style="1" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="9.33203125" style="2" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="11.1640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="20.83203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="15.83203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="8" width="20.83203125" style="1" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="15" style="1" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="8.83203125" customWidth="1"/>
     <col min="11" max="11" width="25.6640625" style="3" bestFit="1" customWidth="1"/>
@@ -2040,16 +2090,16 @@
       </c>
     </row>
     <row r="4" spans="2:14" ht="31" x14ac:dyDescent="0.2">
-      <c r="B4" s="50" t="s">
+      <c r="B4" s="58" t="s">
         <v>9</v>
       </c>
-      <c r="C4" s="50"/>
-      <c r="D4" s="50"/>
-      <c r="E4" s="50"/>
-      <c r="F4" s="50"/>
-      <c r="G4" s="50"/>
-      <c r="H4" s="50"/>
-      <c r="I4" s="50"/>
+      <c r="C4" s="58"/>
+      <c r="D4" s="58"/>
+      <c r="E4" s="58"/>
+      <c r="F4" s="58"/>
+      <c r="G4" s="58"/>
+      <c r="H4" s="58"/>
+      <c r="I4" s="58"/>
       <c r="K4" s="4"/>
       <c r="L4" s="4"/>
       <c r="M4" s="5"/>
@@ -2156,7 +2206,7 @@
       </c>
     </row>
     <row r="11" spans="2:14" ht="17" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B11" s="47" t="s">
+      <c r="B11" s="46" t="s">
         <v>39</v>
       </c>
       <c r="C11" s="19" t="s">
@@ -2241,145 +2291,125 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="B17" s="1" t="s">
+    <row r="17" spans="1:20" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A17" s="1"/>
+      <c r="G17" s="3"/>
+      <c r="H17" s="32" t="s">
+        <v>41</v>
+      </c>
+      <c r="I17" s="52" t="s">
+        <v>43</v>
+      </c>
+      <c r="J17" s="3"/>
+    </row>
+    <row r="18" spans="1:20" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A18" s="1"/>
+      <c r="G18" s="3"/>
+      <c r="H18" s="32" t="s">
+        <v>42</v>
+      </c>
+      <c r="I18" s="52" t="s">
+        <v>44</v>
+      </c>
+      <c r="J18" s="3"/>
+    </row>
+    <row r="19" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="B19" s="1" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="18" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="B18" s="51" t="s">
+    <row r="20" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="B20" s="59" t="s">
         <v>24</v>
       </c>
-      <c r="C18" s="51"/>
-      <c r="D18" s="35" t="e">
+      <c r="C20" s="59"/>
+      <c r="D20" s="35" t="e">
         <f>EDATE(I6,1)</f>
         <v>#VALUE!</v>
       </c>
-      <c r="F18" s="2" t="s">
+      <c r="F20" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="G18" s="1" t="s">
+      <c r="G20" s="1" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="19" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="B19" s="34" t="s">
+    <row r="21" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="B21" s="34" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="20" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="B20" s="52" t="s">
+    <row r="22" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="B22" s="60" t="s">
         <v>27</v>
       </c>
-      <c r="C20" s="52"/>
-      <c r="D20" s="52"/>
-      <c r="E20" s="52"/>
-      <c r="F20" s="52"/>
-      <c r="G20" s="52"/>
-      <c r="H20" s="52"/>
-      <c r="I20" s="52"/>
-    </row>
-    <row r="21" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="B21" s="52" t="s">
+      <c r="C22" s="60"/>
+      <c r="D22" s="60"/>
+      <c r="E22" s="60"/>
+      <c r="F22" s="60"/>
+      <c r="G22" s="60"/>
+      <c r="H22" s="60"/>
+      <c r="I22" s="60"/>
+    </row>
+    <row r="23" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="B23" s="60" t="s">
         <v>28</v>
       </c>
-      <c r="C21" s="52"/>
-      <c r="D21" s="52"/>
-      <c r="E21" s="52"/>
-      <c r="F21" s="52"/>
-      <c r="G21" s="52"/>
-      <c r="H21" s="52"/>
-      <c r="I21" s="52"/>
-    </row>
-    <row r="22" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="B22" s="52" t="s">
+      <c r="C23" s="60"/>
+      <c r="D23" s="60"/>
+      <c r="E23" s="60"/>
+      <c r="F23" s="60"/>
+      <c r="G23" s="60"/>
+      <c r="H23" s="60"/>
+      <c r="I23" s="60"/>
+    </row>
+    <row r="24" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="B24" s="60" t="s">
         <v>29</v>
       </c>
-      <c r="C22" s="52"/>
-      <c r="D22" s="52"/>
-      <c r="E22" s="52"/>
-      <c r="F22" s="52"/>
-      <c r="G22" s="52"/>
-      <c r="H22" s="52"/>
-      <c r="I22" s="52"/>
-    </row>
-    <row r="23" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="B23" s="52" t="s">
+      <c r="C24" s="60"/>
+      <c r="D24" s="60"/>
+      <c r="E24" s="60"/>
+      <c r="F24" s="60"/>
+      <c r="G24" s="60"/>
+      <c r="H24" s="60"/>
+      <c r="I24" s="60"/>
+    </row>
+    <row r="25" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="B25" s="60" t="s">
         <v>30</v>
       </c>
-      <c r="C23" s="52"/>
-      <c r="D23" s="52"/>
-      <c r="E23" s="52"/>
-      <c r="F23" s="52"/>
-      <c r="G23" s="52"/>
-      <c r="H23" s="52"/>
-      <c r="I23" s="52"/>
-    </row>
-    <row r="24" spans="1:20" ht="21" x14ac:dyDescent="0.2">
-      <c r="B24" s="36" t="s">
+      <c r="C25" s="60"/>
+      <c r="D25" s="60"/>
+      <c r="E25" s="60"/>
+      <c r="F25" s="60"/>
+      <c r="G25" s="60"/>
+      <c r="H25" s="60"/>
+      <c r="I25" s="60"/>
+    </row>
+    <row r="26" spans="1:20" ht="21" x14ac:dyDescent="0.2">
+      <c r="B26" s="36" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="25" spans="1:20" ht="21" x14ac:dyDescent="0.2">
-      <c r="B25" s="36" t="s">
+    <row r="27" spans="1:20" ht="21" x14ac:dyDescent="0.2">
+      <c r="B27" s="36" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="26" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="B26" s="34"/>
-      <c r="H26" s="10" t="s">
+    <row r="28" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="B28" s="34"/>
+      <c r="H28" s="10" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="27" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="B27" s="37"/>
-      <c r="H27" s="10" t="s">
+    <row r="29" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="B29" s="37"/>
+      <c r="H29" s="10" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="28" spans="1:20" customFormat="1" ht="74.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A28" s="3"/>
-      <c r="B28" s="37"/>
-      <c r="C28" s="1"/>
-      <c r="D28" s="1"/>
-      <c r="E28" s="2"/>
-      <c r="F28" s="1"/>
-      <c r="G28" s="1"/>
-      <c r="H28" s="10"/>
-      <c r="I28" s="1"/>
-      <c r="K28" s="3"/>
-      <c r="L28" s="3"/>
-      <c r="M28" s="3"/>
-      <c r="N28" s="3"/>
-      <c r="O28" s="3"/>
-      <c r="P28" s="3"/>
-      <c r="Q28" s="3"/>
-      <c r="R28" s="3"/>
-      <c r="S28" s="3"/>
-      <c r="T28" s="3"/>
-    </row>
-    <row r="29" spans="1:20" customFormat="1" ht="16" x14ac:dyDescent="0.2">
-      <c r="A29" s="3"/>
-      <c r="B29" s="48"/>
-      <c r="C29" s="48"/>
-      <c r="D29" s="48"/>
-      <c r="E29" s="48"/>
-      <c r="F29" s="48"/>
-      <c r="G29" s="48"/>
-      <c r="H29" s="48"/>
-      <c r="I29" s="48"/>
-      <c r="K29" s="3"/>
-      <c r="L29" s="3"/>
-      <c r="M29" s="3"/>
-      <c r="N29" s="3"/>
-      <c r="O29" s="3"/>
-      <c r="P29" s="3"/>
-      <c r="Q29" s="3"/>
-      <c r="R29" s="3"/>
-      <c r="S29" s="3"/>
-      <c r="T29" s="3"/>
-    </row>
-    <row r="30" spans="1:20" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:20" customFormat="1" ht="74.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="3"/>
       <c r="B30" s="37"/>
       <c r="C30" s="1"/>
@@ -2400,58 +2430,58 @@
       <c r="S30" s="3"/>
       <c r="T30" s="3"/>
     </row>
-    <row r="33" spans="1:20" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A33" s="3"/>
-      <c r="B33" s="1"/>
-      <c r="C33" s="49"/>
-      <c r="D33" s="49"/>
-      <c r="E33" s="49"/>
-      <c r="F33" s="49"/>
-      <c r="G33" s="49"/>
-      <c r="H33" s="49"/>
-      <c r="I33" s="49"/>
-      <c r="K33" s="3"/>
-      <c r="L33" s="3"/>
-      <c r="M33" s="3"/>
-      <c r="N33" s="3"/>
-      <c r="O33" s="3"/>
-      <c r="P33" s="3"/>
-      <c r="Q33" s="3"/>
-      <c r="R33" s="3"/>
-      <c r="S33" s="3"/>
-      <c r="T33" s="3"/>
-    </row>
-    <row r="34" spans="1:20" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A34" s="3"/>
-      <c r="B34" s="1"/>
-      <c r="C34" s="49"/>
-      <c r="D34" s="49"/>
-      <c r="E34" s="49"/>
-      <c r="F34" s="49"/>
-      <c r="G34" s="49"/>
-      <c r="H34" s="49"/>
-      <c r="I34" s="1"/>
-      <c r="K34" s="3"/>
-      <c r="L34" s="3"/>
-      <c r="M34" s="3"/>
-      <c r="N34" s="3"/>
-      <c r="O34" s="3"/>
-      <c r="P34" s="3"/>
-      <c r="Q34" s="3"/>
-      <c r="R34" s="3"/>
-      <c r="S34" s="3"/>
-      <c r="T34" s="3"/>
+    <row r="31" spans="1:20" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+      <c r="A31" s="3"/>
+      <c r="B31" s="57"/>
+      <c r="C31" s="57"/>
+      <c r="D31" s="57"/>
+      <c r="E31" s="57"/>
+      <c r="F31" s="57"/>
+      <c r="G31" s="57"/>
+      <c r="H31" s="57"/>
+      <c r="I31" s="57"/>
+      <c r="K31" s="3"/>
+      <c r="L31" s="3"/>
+      <c r="M31" s="3"/>
+      <c r="N31" s="3"/>
+      <c r="O31" s="3"/>
+      <c r="P31" s="3"/>
+      <c r="Q31" s="3"/>
+      <c r="R31" s="3"/>
+      <c r="S31" s="3"/>
+      <c r="T31" s="3"/>
+    </row>
+    <row r="32" spans="1:20" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A32" s="3"/>
+      <c r="B32" s="37"/>
+      <c r="C32" s="1"/>
+      <c r="D32" s="1"/>
+      <c r="E32" s="2"/>
+      <c r="F32" s="1"/>
+      <c r="G32" s="1"/>
+      <c r="H32" s="10"/>
+      <c r="I32" s="1"/>
+      <c r="K32" s="3"/>
+      <c r="L32" s="3"/>
+      <c r="M32" s="3"/>
+      <c r="N32" s="3"/>
+      <c r="O32" s="3"/>
+      <c r="P32" s="3"/>
+      <c r="Q32" s="3"/>
+      <c r="R32" s="3"/>
+      <c r="S32" s="3"/>
+      <c r="T32" s="3"/>
     </row>
     <row r="35" spans="1:20" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A35" s="3"/>
       <c r="B35" s="1"/>
-      <c r="C35" s="49"/>
-      <c r="D35" s="49"/>
-      <c r="E35" s="49"/>
-      <c r="F35" s="49"/>
-      <c r="G35" s="49"/>
-      <c r="H35" s="49"/>
-      <c r="I35" s="1"/>
+      <c r="C35" s="53"/>
+      <c r="D35" s="53"/>
+      <c r="E35" s="53"/>
+      <c r="F35" s="53"/>
+      <c r="G35" s="53"/>
+      <c r="H35" s="53"/>
+      <c r="I35" s="53"/>
       <c r="K35" s="3"/>
       <c r="L35" s="3"/>
       <c r="M35" s="3"/>
@@ -2463,22 +2493,64 @@
       <c r="S35" s="3"/>
       <c r="T35" s="3"/>
     </row>
+    <row r="36" spans="1:20" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A36" s="3"/>
+      <c r="B36" s="1"/>
+      <c r="C36" s="53"/>
+      <c r="D36" s="53"/>
+      <c r="E36" s="53"/>
+      <c r="F36" s="53"/>
+      <c r="G36" s="53"/>
+      <c r="H36" s="53"/>
+      <c r="I36" s="1"/>
+      <c r="K36" s="3"/>
+      <c r="L36" s="3"/>
+      <c r="M36" s="3"/>
+      <c r="N36" s="3"/>
+      <c r="O36" s="3"/>
+      <c r="P36" s="3"/>
+      <c r="Q36" s="3"/>
+      <c r="R36" s="3"/>
+      <c r="S36" s="3"/>
+      <c r="T36" s="3"/>
+    </row>
+    <row r="37" spans="1:20" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A37" s="3"/>
+      <c r="B37" s="1"/>
+      <c r="C37" s="53"/>
+      <c r="D37" s="53"/>
+      <c r="E37" s="53"/>
+      <c r="F37" s="53"/>
+      <c r="G37" s="53"/>
+      <c r="H37" s="53"/>
+      <c r="I37" s="1"/>
+      <c r="K37" s="3"/>
+      <c r="L37" s="3"/>
+      <c r="M37" s="3"/>
+      <c r="N37" s="3"/>
+      <c r="O37" s="3"/>
+      <c r="P37" s="3"/>
+      <c r="Q37" s="3"/>
+      <c r="R37" s="3"/>
+      <c r="S37" s="3"/>
+      <c r="T37" s="3"/>
+    </row>
   </sheetData>
   <mergeCells count="10">
-    <mergeCell ref="B29:I29"/>
-    <mergeCell ref="C33:I33"/>
-    <mergeCell ref="C34:H34"/>
-    <mergeCell ref="C35:H35"/>
+    <mergeCell ref="B31:I31"/>
+    <mergeCell ref="C35:I35"/>
+    <mergeCell ref="C36:H36"/>
+    <mergeCell ref="C37:H37"/>
     <mergeCell ref="B4:I4"/>
-    <mergeCell ref="B18:C18"/>
-    <mergeCell ref="B20:I20"/>
-    <mergeCell ref="B21:I21"/>
+    <mergeCell ref="B20:C20"/>
     <mergeCell ref="B22:I22"/>
     <mergeCell ref="B23:I23"/>
+    <mergeCell ref="B24:I24"/>
+    <mergeCell ref="B25:I25"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="3.937007874015748E-2" right="3.937007874015748E-2" top="0.39370078740157483" bottom="0.19685039370078741" header="0.39370078740157483" footer="0"/>
-  <pageSetup paperSize="9" scale="76" orientation="portrait" r:id="rId1"/>
+  <pageSetup paperSize="9" scale="73" orientation="portrait" r:id="rId1"/>
   <headerFooter>
     <oddHeader>&amp;C&amp;G</oddHeader>
     <oddFooter>&amp;C&amp;G</oddFooter>
@@ -2495,7 +2567,7 @@
   <sheetPr codeName="Sheet9">
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:T25"/>
+  <dimension ref="A1:T27"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.1640625" defaultRowHeight="20" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="2.5" style="1" customWidth="1"/>
@@ -2529,19 +2601,19 @@
       </c>
     </row>
     <row r="4" spans="1:14" ht="31" x14ac:dyDescent="0.2">
-      <c r="B4" s="53" t="s">
+      <c r="B4" s="54" t="s">
         <v>33</v>
       </c>
-      <c r="C4" s="53"/>
-      <c r="D4" s="53"/>
-      <c r="E4" s="53"/>
-      <c r="F4" s="53"/>
-      <c r="G4" s="53"/>
-      <c r="H4" s="53"/>
-      <c r="I4" s="53"/>
-      <c r="J4" s="53"/>
-      <c r="K4" s="53"/>
-      <c r="L4" s="53"/>
+      <c r="C4" s="54"/>
+      <c r="D4" s="54"/>
+      <c r="E4" s="54"/>
+      <c r="F4" s="54"/>
+      <c r="G4" s="54"/>
+      <c r="H4" s="54"/>
+      <c r="I4" s="54"/>
+      <c r="J4" s="54"/>
+      <c r="K4" s="54"/>
+      <c r="L4" s="54"/>
       <c r="M4" s="5"/>
       <c r="N4" s="6"/>
     </row>
@@ -2651,7 +2723,7 @@
       </c>
     </row>
     <row r="11" spans="1:14" ht="17" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B11" s="47" t="s">
+      <c r="B11" s="46" t="s">
         <v>40</v>
       </c>
       <c r="C11" s="19"/>
@@ -2668,120 +2740,100 @@
       <c r="N11" s="43"/>
     </row>
     <row r="12" spans="1:14" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="G12" s="32" t="s">
+      <c r="G12" s="47" t="s">
         <v>23</v>
       </c>
-      <c r="H12" s="24" t="s">
+      <c r="H12" s="48" t="s">
         <v>19</v>
       </c>
-      <c r="I12" s="25">
+      <c r="I12" s="49">
         <f>SUM(I11:I11)</f>
         <v>0</v>
       </c>
-      <c r="J12" s="25">
+      <c r="J12" s="49">
         <f>SUM(J11:J11)</f>
         <v>0</v>
       </c>
       <c r="K12" s="44" t="s">
         <v>20</v>
       </c>
-      <c r="L12" s="45">
+      <c r="L12" s="50">
         <f>SUM(L11:L11)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:14" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="H13" s="23" t="s">
+    <row r="13" spans="1:14" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="G13" s="32" t="s">
+        <v>41</v>
+      </c>
+      <c r="H13" s="32"/>
+      <c r="I13" s="51"/>
+      <c r="J13" s="51"/>
+      <c r="K13" s="32"/>
+      <c r="L13" s="52" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="14" spans="1:14" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="G14" s="32" t="s">
+        <v>42</v>
+      </c>
+      <c r="H14" s="32"/>
+      <c r="I14" s="51"/>
+      <c r="J14" s="51"/>
+      <c r="K14" s="32"/>
+      <c r="L14" s="52" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="15" spans="1:14" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="H15" s="23" t="s">
         <v>22</v>
       </c>
-      <c r="I13" s="31">
+      <c r="I15" s="31">
         <f>I12*18%</f>
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:14" ht="210.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B14" s="54" t="s">
+    <row r="16" spans="1:14" ht="210.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B16" s="55" t="s">
         <v>34</v>
       </c>
-      <c r="C14" s="54"/>
-      <c r="D14" s="54"/>
-      <c r="E14" s="54"/>
-      <c r="F14" s="54"/>
-      <c r="G14" s="54"/>
-      <c r="H14" s="54"/>
-      <c r="I14" s="54"/>
-      <c r="J14" s="54"/>
-      <c r="K14" s="54"/>
-      <c r="L14" s="54"/>
-    </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="E15" s="1"/>
-      <c r="F15" s="55" t="s">
+      <c r="C16" s="55"/>
+      <c r="D16" s="55"/>
+      <c r="E16" s="55"/>
+      <c r="F16" s="55"/>
+      <c r="G16" s="55"/>
+      <c r="H16" s="55"/>
+      <c r="I16" s="55"/>
+      <c r="J16" s="55"/>
+      <c r="K16" s="55"/>
+      <c r="L16" s="55"/>
+    </row>
+    <row r="17" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="E17" s="1"/>
+      <c r="F17" s="56" t="s">
         <v>35</v>
       </c>
-      <c r="G15" s="55"/>
-      <c r="J15" s="1"/>
-    </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="B16" s="46"/>
-      <c r="C16" s="46"/>
-      <c r="D16" s="46"/>
-      <c r="E16" s="46"/>
-      <c r="F16" s="10"/>
-      <c r="G16" s="46"/>
-      <c r="H16" s="46"/>
-      <c r="I16" s="46"/>
-      <c r="J16" s="1"/>
-    </row>
-    <row r="17" spans="1:20" ht="78" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B17" s="37"/>
-      <c r="E17" s="1"/>
-      <c r="F17" s="10"/>
+      <c r="G17" s="56"/>
       <c r="J17" s="1"/>
     </row>
-    <row r="18" spans="1:20" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A18" s="38"/>
-      <c r="B18" s="37"/>
-      <c r="C18" s="1"/>
-      <c r="D18" s="1"/>
-      <c r="E18" s="2"/>
-      <c r="F18" s="1"/>
-      <c r="G18" s="1"/>
-      <c r="H18" s="10"/>
-      <c r="I18" s="1"/>
-      <c r="J18" s="38"/>
-      <c r="K18" s="1"/>
-      <c r="L18" s="1"/>
-      <c r="M18" s="3"/>
-      <c r="N18" s="3"/>
-      <c r="O18" s="3"/>
-      <c r="P18" s="3"/>
-      <c r="Q18" s="3"/>
-      <c r="R18" s="3"/>
-      <c r="S18" s="3"/>
-      <c r="T18" s="3"/>
-    </row>
-    <row r="19" spans="1:20" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A19" s="38"/>
-      <c r="B19" s="48"/>
-      <c r="C19" s="48"/>
-      <c r="D19" s="48"/>
-      <c r="E19" s="48"/>
-      <c r="F19" s="48"/>
-      <c r="G19" s="48"/>
-      <c r="H19" s="48"/>
-      <c r="I19" s="48"/>
-      <c r="J19" s="38"/>
-      <c r="K19" s="1"/>
-      <c r="L19" s="1"/>
-      <c r="M19" s="3"/>
-      <c r="N19" s="3"/>
-      <c r="O19" s="3"/>
-      <c r="P19" s="3"/>
-      <c r="Q19" s="3"/>
-      <c r="R19" s="3"/>
-      <c r="S19" s="3"/>
-      <c r="T19" s="3"/>
+    <row r="18" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="B18" s="45"/>
+      <c r="C18" s="45"/>
+      <c r="D18" s="45"/>
+      <c r="E18" s="45"/>
+      <c r="F18" s="10"/>
+      <c r="G18" s="45"/>
+      <c r="H18" s="45"/>
+      <c r="I18" s="45"/>
+      <c r="J18" s="1"/>
+    </row>
+    <row r="19" spans="1:20" ht="78" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B19" s="37"/>
+      <c r="E19" s="1"/>
+      <c r="F19" s="10"/>
+      <c r="J19" s="1"/>
     </row>
     <row r="20" spans="1:20" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A20" s="38"/>
@@ -2805,60 +2857,60 @@
       <c r="S20" s="3"/>
       <c r="T20" s="3"/>
     </row>
-    <row r="23" spans="1:20" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A23" s="38"/>
-      <c r="B23" s="1"/>
-      <c r="C23" s="49"/>
-      <c r="D23" s="49"/>
-      <c r="E23" s="49"/>
-      <c r="F23" s="49"/>
-      <c r="G23" s="49"/>
-      <c r="H23" s="49"/>
-      <c r="I23" s="49"/>
-      <c r="J23" s="38"/>
-      <c r="K23" s="1"/>
-      <c r="L23" s="1"/>
-      <c r="M23" s="3"/>
-      <c r="N23" s="3"/>
-      <c r="O23" s="3"/>
-      <c r="P23" s="3"/>
-      <c r="Q23" s="3"/>
-      <c r="R23" s="3"/>
-      <c r="S23" s="3"/>
-      <c r="T23" s="3"/>
-    </row>
-    <row r="24" spans="1:20" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A24" s="38"/>
-      <c r="B24" s="1"/>
-      <c r="C24" s="49"/>
-      <c r="D24" s="49"/>
-      <c r="E24" s="49"/>
-      <c r="F24" s="49"/>
-      <c r="G24" s="49"/>
-      <c r="H24" s="49"/>
-      <c r="I24" s="1"/>
-      <c r="J24" s="38"/>
-      <c r="K24" s="1"/>
-      <c r="L24" s="1"/>
-      <c r="M24" s="3"/>
-      <c r="N24" s="3"/>
-      <c r="O24" s="3"/>
-      <c r="P24" s="3"/>
-      <c r="Q24" s="3"/>
-      <c r="R24" s="3"/>
-      <c r="S24" s="3"/>
-      <c r="T24" s="3"/>
+    <row r="21" spans="1:20" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A21" s="38"/>
+      <c r="B21" s="57"/>
+      <c r="C21" s="57"/>
+      <c r="D21" s="57"/>
+      <c r="E21" s="57"/>
+      <c r="F21" s="57"/>
+      <c r="G21" s="57"/>
+      <c r="H21" s="57"/>
+      <c r="I21" s="57"/>
+      <c r="J21" s="38"/>
+      <c r="K21" s="1"/>
+      <c r="L21" s="1"/>
+      <c r="M21" s="3"/>
+      <c r="N21" s="3"/>
+      <c r="O21" s="3"/>
+      <c r="P21" s="3"/>
+      <c r="Q21" s="3"/>
+      <c r="R21" s="3"/>
+      <c r="S21" s="3"/>
+      <c r="T21" s="3"/>
+    </row>
+    <row r="22" spans="1:20" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A22" s="38"/>
+      <c r="B22" s="37"/>
+      <c r="C22" s="1"/>
+      <c r="D22" s="1"/>
+      <c r="E22" s="2"/>
+      <c r="F22" s="1"/>
+      <c r="G22" s="1"/>
+      <c r="H22" s="10"/>
+      <c r="I22" s="1"/>
+      <c r="J22" s="38"/>
+      <c r="K22" s="1"/>
+      <c r="L22" s="1"/>
+      <c r="M22" s="3"/>
+      <c r="N22" s="3"/>
+      <c r="O22" s="3"/>
+      <c r="P22" s="3"/>
+      <c r="Q22" s="3"/>
+      <c r="R22" s="3"/>
+      <c r="S22" s="3"/>
+      <c r="T22" s="3"/>
     </row>
     <row r="25" spans="1:20" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A25" s="38"/>
       <c r="B25" s="1"/>
-      <c r="C25" s="49"/>
-      <c r="D25" s="49"/>
-      <c r="E25" s="49"/>
-      <c r="F25" s="49"/>
-      <c r="G25" s="49"/>
-      <c r="H25" s="49"/>
-      <c r="I25" s="1"/>
+      <c r="C25" s="53"/>
+      <c r="D25" s="53"/>
+      <c r="E25" s="53"/>
+      <c r="F25" s="53"/>
+      <c r="G25" s="53"/>
+      <c r="H25" s="53"/>
+      <c r="I25" s="53"/>
       <c r="J25" s="38"/>
       <c r="K25" s="1"/>
       <c r="L25" s="1"/>
@@ -2871,20 +2923,64 @@
       <c r="S25" s="3"/>
       <c r="T25" s="3"/>
     </row>
+    <row r="26" spans="1:20" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A26" s="38"/>
+      <c r="B26" s="1"/>
+      <c r="C26" s="53"/>
+      <c r="D26" s="53"/>
+      <c r="E26" s="53"/>
+      <c r="F26" s="53"/>
+      <c r="G26" s="53"/>
+      <c r="H26" s="53"/>
+      <c r="I26" s="1"/>
+      <c r="J26" s="38"/>
+      <c r="K26" s="1"/>
+      <c r="L26" s="1"/>
+      <c r="M26" s="3"/>
+      <c r="N26" s="3"/>
+      <c r="O26" s="3"/>
+      <c r="P26" s="3"/>
+      <c r="Q26" s="3"/>
+      <c r="R26" s="3"/>
+      <c r="S26" s="3"/>
+      <c r="T26" s="3"/>
+    </row>
+    <row r="27" spans="1:20" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A27" s="38"/>
+      <c r="B27" s="1"/>
+      <c r="C27" s="53"/>
+      <c r="D27" s="53"/>
+      <c r="E27" s="53"/>
+      <c r="F27" s="53"/>
+      <c r="G27" s="53"/>
+      <c r="H27" s="53"/>
+      <c r="I27" s="1"/>
+      <c r="J27" s="38"/>
+      <c r="K27" s="1"/>
+      <c r="L27" s="1"/>
+      <c r="M27" s="3"/>
+      <c r="N27" s="3"/>
+      <c r="O27" s="3"/>
+      <c r="P27" s="3"/>
+      <c r="Q27" s="3"/>
+      <c r="R27" s="3"/>
+      <c r="S27" s="3"/>
+      <c r="T27" s="3"/>
+    </row>
   </sheetData>
   <mergeCells count="7">
-    <mergeCell ref="C25:H25"/>
+    <mergeCell ref="C27:H27"/>
     <mergeCell ref="B4:L4"/>
-    <mergeCell ref="B14:L14"/>
-    <mergeCell ref="F15:G15"/>
-    <mergeCell ref="B19:I19"/>
-    <mergeCell ref="C23:I23"/>
-    <mergeCell ref="C24:H24"/>
+    <mergeCell ref="B16:L16"/>
+    <mergeCell ref="F17:G17"/>
+    <mergeCell ref="B21:I21"/>
+    <mergeCell ref="C25:I25"/>
+    <mergeCell ref="C26:H26"/>
   </mergeCells>
   <phoneticPr fontId="19" type="noConversion"/>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="3.937007874015748E-2" right="3.937007874015748E-2" top="0.39370078740157483" bottom="0.19685039370078741" header="0.39370078740157483" footer="0"/>
-  <pageSetup paperSize="9" scale="87" orientation="portrait" r:id="rId1"/>
+  <pageSetup paperSize="9" scale="86" orientation="portrait" r:id="rId1"/>
   <headerFooter>
     <oddHeader>&amp;C&amp;G</oddHeader>
     <oddFooter>&amp;C&amp;G</oddFooter>

</xml_diff>

<commit_message>
feat(discount): per-user client discount applied to price proposal
Admin sets a nullable discount_percent (0–100) per user in the Users tab;
null means normal price. The proposal generator looks up the project
owner's discount and resolves the PRICE_AFTER_DISCOUNT token (at I13) to
=<cell above>*(100-d)/100, or =<cell above> when null — flowing through
the VAT/total chain. References are relative to the token's final row, so
they stay correct as BOM rows shift the totals block down.

- users.discount_percent column + alembic 0052
- UserRead/UserUpdate schemas (0–100 validation)
- admin update_user: exclude_unset so an explicit null can clear it
- Users tab: editable Discount % column + en/he labels

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BE/mgp-service/app/templates/proposal_template.xlsx
+++ b/BE/mgp-service/app/templates/proposal_template.xlsx
@@ -1,9 +1,9 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10503"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10517"/>
   <workbookPr filterPrivacy="1" codeName="ThisWorkbook"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B5A6DDC3-89D5-364A-ADEE-326CDD5EB49F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0AFCCE0E-96C9-6744-A775-1C44AB45814B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="19720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="46">
   <si>
     <t>שורה</t>
   </si>
@@ -184,6 +184,9 @@
   </si>
   <si>
     <t>ALUMINIUM_WEIGHT</t>
+  </si>
+  <si>
+    <t>PRICE_AFTER_DISCOUNT</t>
   </si>
 </sst>
 </file>
@@ -573,9 +576,21 @@
     <xf numFmtId="165" fontId="18" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" readingOrder="2"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" readingOrder="2"/>
     </xf>
@@ -584,18 +599,6 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" readingOrder="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" readingOrder="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" readingOrder="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -616,8 +619,25 @@
         <vertAlign val="baseline"/>
         <sz val="12"/>
         <color rgb="FF000000"/>
-        <name val="Calibri"/>
-        <family val="2"/>
+        <name val="Heebo"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <name val="Heebo"/>
         <scheme val="none"/>
       </font>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -654,8 +674,7 @@
         <vertAlign val="baseline"/>
         <sz val="12"/>
         <color rgb="FF000000"/>
-        <name val="Calibri"/>
-        <family val="2"/>
+        <name val="Heebo"/>
         <scheme val="none"/>
       </font>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -692,10 +711,10 @@
         <vertAlign val="baseline"/>
         <sz val="12"/>
         <color rgb="FF000000"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
+        <name val="Heebo"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="4" formatCode="#,##0.00"/>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
@@ -730,71 +749,12 @@
         <vertAlign val="baseline"/>
         <sz val="12"/>
         <color rgb="FF000000"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <name val="Calibri"/>
-        <family val="2"/>
+        <name val="Heebo"/>
         <scheme val="none"/>
       </font>
       <numFmt numFmtId="4" formatCode="#,##0.00"/>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="4" formatCode="#,##0.00"/>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
+      <border diagonalUp="0" diagonalDown="0" outline="0">
         <left style="thin">
           <color indexed="64"/>
         </left>
@@ -807,12 +767,6 @@
         <bottom style="thin">
           <color indexed="64"/>
         </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
       </border>
     </dxf>
     <dxf>
@@ -884,6 +838,7 @@
         <strike val="0"/>
         <outline val="0"/>
         <shadow val="0"/>
+        <u val="none"/>
         <vertAlign val="baseline"/>
         <sz val="12"/>
         <name val="Heebo"/>
@@ -910,6 +865,7 @@
         <strike val="0"/>
         <outline val="0"/>
         <shadow val="0"/>
+        <u val="none"/>
         <vertAlign val="baseline"/>
         <sz val="12"/>
         <name val="Heebo"/>
@@ -935,6 +891,7 @@
         <strike val="0"/>
         <outline val="0"/>
         <shadow val="0"/>
+        <u val="none"/>
         <vertAlign val="baseline"/>
         <sz val="12"/>
         <name val="Heebo"/>
@@ -1025,6 +982,7 @@
         <strike val="0"/>
         <outline val="0"/>
         <shadow val="0"/>
+        <u val="none"/>
         <vertAlign val="baseline"/>
         <sz val="12"/>
         <name val="Heebo"/>
@@ -1100,8 +1058,7 @@
         <vertAlign val="baseline"/>
         <sz val="12"/>
         <color rgb="FF000000"/>
-        <name val="Calibri"/>
-        <family val="2"/>
+        <name val="Heebo"/>
         <scheme val="none"/>
       </font>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -1126,9 +1083,8 @@
         <vertAlign val="baseline"/>
         <sz val="12"/>
         <color theme="0"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
+        <name val="Heebo"/>
+        <scheme val="none"/>
       </font>
       <fill>
         <patternFill patternType="solid">
@@ -1161,25 +1117,8 @@
         <vertAlign val="baseline"/>
         <sz val="12"/>
         <color rgb="FF000000"/>
-        <name val="Heebo"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <name val="Heebo"/>
+        <name val="Calibri"/>
+        <family val="2"/>
         <scheme val="none"/>
       </font>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -1216,7 +1155,8 @@
         <vertAlign val="baseline"/>
         <sz val="12"/>
         <color rgb="FF000000"/>
-        <name val="Heebo"/>
+        <name val="Calibri"/>
+        <family val="2"/>
         <scheme val="none"/>
       </font>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -1253,10 +1193,10 @@
         <vertAlign val="baseline"/>
         <sz val="12"/>
         <color rgb="FF000000"/>
-        <name val="Heebo"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="4" formatCode="#,##0.00"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
@@ -1291,12 +1231,71 @@
         <vertAlign val="baseline"/>
         <sz val="12"/>
         <color rgb="FF000000"/>
-        <name val="Heebo"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <name val="Calibri"/>
+        <family val="2"/>
         <scheme val="none"/>
       </font>
       <numFmt numFmtId="4" formatCode="#,##0.00"/>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="4" formatCode="#,##0.00"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
         <left style="thin">
           <color indexed="64"/>
         </left>
@@ -1309,6 +1308,12 @@
         <bottom style="thin">
           <color indexed="64"/>
         </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
       </border>
     </dxf>
     <dxf>
@@ -1380,7 +1385,6 @@
         <strike val="0"/>
         <outline val="0"/>
         <shadow val="0"/>
-        <u val="none"/>
         <vertAlign val="baseline"/>
         <sz val="12"/>
         <name val="Heebo"/>
@@ -1407,7 +1411,6 @@
         <strike val="0"/>
         <outline val="0"/>
         <shadow val="0"/>
-        <u val="none"/>
         <vertAlign val="baseline"/>
         <sz val="12"/>
         <name val="Heebo"/>
@@ -1433,7 +1436,6 @@
         <strike val="0"/>
         <outline val="0"/>
         <shadow val="0"/>
-        <u val="none"/>
         <vertAlign val="baseline"/>
         <sz val="12"/>
         <name val="Heebo"/>
@@ -1524,7 +1526,6 @@
         <strike val="0"/>
         <outline val="0"/>
         <shadow val="0"/>
-        <u val="none"/>
         <vertAlign val="baseline"/>
         <sz val="12"/>
         <name val="Heebo"/>
@@ -1600,7 +1601,8 @@
         <vertAlign val="baseline"/>
         <sz val="12"/>
         <color rgb="FF000000"/>
-        <name val="Heebo"/>
+        <name val="Calibri"/>
+        <family val="2"/>
         <scheme val="none"/>
       </font>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -1625,8 +1627,9 @@
         <vertAlign val="baseline"/>
         <sz val="12"/>
         <color theme="0"/>
-        <name val="Heebo"/>
-        <scheme val="none"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
       </font>
       <fill>
         <patternFill patternType="solid">
@@ -1683,48 +1686,48 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{5ACB1EC1-21C6-AF40-A140-308C9117B91F}" name="pricing_table25" displayName="pricing_table25" ref="B10:N11" totalsRowShown="0" headerRowDxfId="23" dataDxfId="21" totalsRowDxfId="19" headerRowBorderDxfId="22" tableBorderDxfId="20" totalsRowBorderDxfId="18">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{5ACB1EC1-21C6-AF40-A140-308C9117B91F}" name="pricing_table25" displayName="pricing_table25" ref="B10:N11" totalsRowShown="0" headerRowDxfId="45" dataDxfId="43" totalsRowDxfId="41" headerRowBorderDxfId="44" tableBorderDxfId="42" totalsRowBorderDxfId="40">
   <autoFilter ref="B10:N11" xr:uid="{A700047D-2A12-4A24-87A3-5C54C0CD36D6}"/>
   <tableColumns count="13">
-    <tableColumn id="1" xr3:uid="{9715C0F5-6C58-0C48-A92D-3904FFEE1286}" name="שורה" dataDxfId="17"/>
-    <tableColumn id="2" xr3:uid="{E71665ED-EE05-B544-8402-B3336F34DA2C}" name="מיקום בגג" dataDxfId="16"/>
-    <tableColumn id="3" xr3:uid="{58C96AFC-B01E-D446-8E2A-ACF7B2497559}" name="תאור מוצר" dataDxfId="15"/>
-    <tableColumn id="4" xr3:uid="{D9DC81BB-9F60-0047-86B9-14278D4E2EE7}" name="אורך" dataDxfId="14"/>
-    <tableColumn id="5" xr3:uid="{B9B74024-7469-A149-9639-A328A6F77916}" name="כמות" dataDxfId="13"/>
-    <tableColumn id="6" xr3:uid="{0FF2A4DA-EE5D-564C-892E-1BAF5895A4E7}" name="כמות: ק&quot;ג\יחידות" dataDxfId="12"/>
-    <tableColumn id="7" xr3:uid="{D3D78E52-A52E-C949-9ABD-03AD0269F0BF}" name="מחיר ליחידה (₪)" dataDxfId="11"/>
-    <tableColumn id="8" xr3:uid="{E1EB6162-FB78-1D4F-9435-2CE9366E3552}" name="סה&quot;כ מחיר (₪)" dataDxfId="10">
+    <tableColumn id="1" xr3:uid="{9715C0F5-6C58-0C48-A92D-3904FFEE1286}" name="שורה" dataDxfId="39"/>
+    <tableColumn id="2" xr3:uid="{E71665ED-EE05-B544-8402-B3336F34DA2C}" name="מיקום בגג" dataDxfId="38"/>
+    <tableColumn id="3" xr3:uid="{58C96AFC-B01E-D446-8E2A-ACF7B2497559}" name="תאור מוצר" dataDxfId="37"/>
+    <tableColumn id="4" xr3:uid="{D9DC81BB-9F60-0047-86B9-14278D4E2EE7}" name="אורך" dataDxfId="36"/>
+    <tableColumn id="5" xr3:uid="{B9B74024-7469-A149-9639-A328A6F77916}" name="כמות" dataDxfId="35"/>
+    <tableColumn id="6" xr3:uid="{0FF2A4DA-EE5D-564C-892E-1BAF5895A4E7}" name="כמות: ק&quot;ג\יחידות" dataDxfId="34"/>
+    <tableColumn id="7" xr3:uid="{D3D78E52-A52E-C949-9ABD-03AD0269F0BF}" name="מחיר ליחידה (₪)" dataDxfId="33"/>
+    <tableColumn id="8" xr3:uid="{E1EB6162-FB78-1D4F-9435-2CE9366E3552}" name="סה&quot;כ מחיר (₪)" dataDxfId="32">
       <calculatedColumnFormula>pricing_table25[[#This Row],[מחיר ליחידה (₪)]]*pricing_table25[[#This Row],[כמות: ק"ג\יחידות]]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{EAED02B8-7E3B-9B47-8C95-FD7B3D6B7DA0}" name="*כמות פחת" dataDxfId="9" totalsRowDxfId="8"/>
-    <tableColumn id="10" xr3:uid="{8DD3D515-E5F7-3F44-AEEC-EBD82CE3FE68}" name="סה&quot;כ מחיר כולל פחת (₪)" dataDxfId="7" totalsRowDxfId="6"/>
-    <tableColumn id="11" xr3:uid="{B17131E0-AD15-314F-8745-C01B5B56C8B5}" name="*משקל בק&quot;ג" dataDxfId="5" totalsRowDxfId="4"/>
-    <tableColumn id="12" xr3:uid="{8383AEF5-4B81-5944-B8C1-7A02610AD799}" name="&gt;% Discount - Construction" dataDxfId="3" totalsRowDxfId="2"/>
-    <tableColumn id="13" xr3:uid="{A6FF8C60-F61C-014D-BE3D-D97E0E91917D}" name="*סה&quot;כ מחיר כולל פחת אחרי הנחה (₪)" dataDxfId="1" totalsRowDxfId="0"/>
+    <tableColumn id="9" xr3:uid="{EAED02B8-7E3B-9B47-8C95-FD7B3D6B7DA0}" name="*כמות פחת" dataDxfId="31" totalsRowDxfId="30"/>
+    <tableColumn id="10" xr3:uid="{8DD3D515-E5F7-3F44-AEEC-EBD82CE3FE68}" name="סה&quot;כ מחיר כולל פחת (₪)" dataDxfId="29" totalsRowDxfId="28"/>
+    <tableColumn id="11" xr3:uid="{B17131E0-AD15-314F-8745-C01B5B56C8B5}" name="*משקל בק&quot;ג" dataDxfId="27" totalsRowDxfId="26"/>
+    <tableColumn id="12" xr3:uid="{8383AEF5-4B81-5944-B8C1-7A02610AD799}" name="&gt;% Discount - Construction" dataDxfId="25" totalsRowDxfId="24"/>
+    <tableColumn id="13" xr3:uid="{A6FF8C60-F61C-014D-BE3D-D97E0E91917D}" name="*סה&quot;כ מחיר כולל פחת אחרי הנחה (₪)" dataDxfId="23" totalsRowDxfId="22"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium15" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{53B791F9-974C-2D45-9198-4628741EC180}" name="pricing_table34" displayName="pricing_table34" ref="B10:N11" totalsRowShown="0" headerRowDxfId="45" dataDxfId="43" totalsRowDxfId="41" headerRowBorderDxfId="44" tableBorderDxfId="42" totalsRowBorderDxfId="40">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{53B791F9-974C-2D45-9198-4628741EC180}" name="pricing_table34" displayName="pricing_table34" ref="B10:N11" totalsRowShown="0" headerRowDxfId="21" dataDxfId="19" totalsRowDxfId="17" headerRowBorderDxfId="20" tableBorderDxfId="18" totalsRowBorderDxfId="16">
   <autoFilter ref="B10:N11" xr:uid="{A700047D-2A12-4A24-87A3-5C54C0CD36D6}"/>
   <tableColumns count="13">
-    <tableColumn id="1" xr3:uid="{C9E84F90-D937-9240-8769-8F47365B79B5}" name="שורה" dataDxfId="39"/>
-    <tableColumn id="2" xr3:uid="{584DEAFB-76D6-C647-A742-316CAAE5BC89}" name="מיקום בגג" dataDxfId="38"/>
-    <tableColumn id="3" xr3:uid="{199A858B-5154-3C42-B14B-B655372B7E72}" name="תאור מוצר" dataDxfId="37"/>
-    <tableColumn id="4" xr3:uid="{044A01A8-0D84-EB4C-A2F1-510AF1F79EC1}" name="אורך" dataDxfId="36"/>
-    <tableColumn id="5" xr3:uid="{23494D31-1003-EC4A-B3E4-56115FE1DC9B}" name="כמות" dataDxfId="35"/>
-    <tableColumn id="6" xr3:uid="{C3ADA01B-011E-AF49-B8EF-BF51E4952D25}" name="כמות: ק&quot;ג\יחידות" dataDxfId="34"/>
-    <tableColumn id="7" xr3:uid="{A4F8123E-37EB-2544-80EC-813AFA9298EC}" name="מחיר ליחידה (₪)" dataDxfId="33"/>
-    <tableColumn id="8" xr3:uid="{891F3848-661F-3446-A7E0-95642AC543B8}" name="סה&quot;כ מחיר (₪)" dataDxfId="32">
+    <tableColumn id="1" xr3:uid="{C9E84F90-D937-9240-8769-8F47365B79B5}" name="שורה" dataDxfId="15"/>
+    <tableColumn id="2" xr3:uid="{584DEAFB-76D6-C647-A742-316CAAE5BC89}" name="מיקום בגג" dataDxfId="14"/>
+    <tableColumn id="3" xr3:uid="{199A858B-5154-3C42-B14B-B655372B7E72}" name="תאור מוצר" dataDxfId="13"/>
+    <tableColumn id="4" xr3:uid="{044A01A8-0D84-EB4C-A2F1-510AF1F79EC1}" name="אורך" dataDxfId="12"/>
+    <tableColumn id="5" xr3:uid="{23494D31-1003-EC4A-B3E4-56115FE1DC9B}" name="כמות" dataDxfId="11"/>
+    <tableColumn id="6" xr3:uid="{C3ADA01B-011E-AF49-B8EF-BF51E4952D25}" name="כמות: ק&quot;ג\יחידות" dataDxfId="10"/>
+    <tableColumn id="7" xr3:uid="{A4F8123E-37EB-2544-80EC-813AFA9298EC}" name="מחיר ליחידה (₪)" dataDxfId="9"/>
+    <tableColumn id="8" xr3:uid="{891F3848-661F-3446-A7E0-95642AC543B8}" name="סה&quot;כ מחיר (₪)" dataDxfId="8">
       <calculatedColumnFormula>pricing_table34[[#This Row],[מחיר ליחידה (₪)]]*pricing_table34[[#This Row],[כמות: ק"ג\יחידות]]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{A50A1AEB-0486-8F4C-A4F6-1B417D72DF83}" name="*כמות פחת" dataDxfId="31" totalsRowDxfId="30"/>
-    <tableColumn id="10" xr3:uid="{3B89E727-3B11-4A40-B717-5C248FA24D57}" name="סה&quot;כ מחיר כולל פחת (₪)" dataDxfId="29" totalsRowDxfId="28"/>
-    <tableColumn id="11" xr3:uid="{981756E0-FF9F-014E-A803-EA2D248E751E}" name="*משקל בק&quot;ג" dataDxfId="27" totalsRowDxfId="26"/>
-    <tableColumn id="12" xr3:uid="{DAD5CC53-679B-024A-96B0-9223C3E03988}" name="&gt;% Discount - Construction" dataDxfId="25"/>
-    <tableColumn id="13" xr3:uid="{7498AF7D-E4AF-4D4F-A51C-BC365E54108A}" name="*סה&quot;כ מחיר כולל פחת אחרי הנחה (₪)" dataDxfId="24"/>
+    <tableColumn id="9" xr3:uid="{A50A1AEB-0486-8F4C-A4F6-1B417D72DF83}" name="*כמות פחת" dataDxfId="7" totalsRowDxfId="6"/>
+    <tableColumn id="10" xr3:uid="{3B89E727-3B11-4A40-B717-5C248FA24D57}" name="סה&quot;כ מחיר כולל פחת (₪)" dataDxfId="5" totalsRowDxfId="4"/>
+    <tableColumn id="11" xr3:uid="{981756E0-FF9F-014E-A803-EA2D248E751E}" name="*משקל בק&quot;ג" dataDxfId="3" totalsRowDxfId="2"/>
+    <tableColumn id="12" xr3:uid="{DAD5CC53-679B-024A-96B0-9223C3E03988}" name="&gt;% Discount - Construction" dataDxfId="1"/>
+    <tableColumn id="13" xr3:uid="{7498AF7D-E4AF-4D4F-A51C-BC365E54108A}" name="*סה&quot;כ מחיר כולל פחת אחרי הנחה (₪)" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium15" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2090,16 +2093,16 @@
       </c>
     </row>
     <row r="4" spans="2:14" ht="31" x14ac:dyDescent="0.2">
-      <c r="B4" s="58" t="s">
+      <c r="B4" s="55" t="s">
         <v>9</v>
       </c>
-      <c r="C4" s="58"/>
-      <c r="D4" s="58"/>
-      <c r="E4" s="58"/>
-      <c r="F4" s="58"/>
-      <c r="G4" s="58"/>
-      <c r="H4" s="58"/>
-      <c r="I4" s="58"/>
+      <c r="C4" s="55"/>
+      <c r="D4" s="55"/>
+      <c r="E4" s="55"/>
+      <c r="F4" s="55"/>
+      <c r="G4" s="55"/>
+      <c r="H4" s="55"/>
+      <c r="I4" s="55"/>
       <c r="K4" s="4"/>
       <c r="L4" s="4"/>
       <c r="M4" s="5"/>
@@ -2255,9 +2258,8 @@
       <c r="H13" s="24" t="s">
         <v>21</v>
       </c>
-      <c r="I13" s="25">
-        <f>N12</f>
-        <v>0</v>
+      <c r="I13" s="52" t="s">
+        <v>45</v>
       </c>
       <c r="J13" s="29"/>
       <c r="K13" s="27"/>
@@ -2268,18 +2270,18 @@
       <c r="H14" s="23" t="s">
         <v>22</v>
       </c>
-      <c r="I14" s="31">
+      <c r="I14" s="31" t="e">
         <f>I13*18%</f>
-        <v>0</v>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="15" spans="2:14" x14ac:dyDescent="0.2">
       <c r="H15" s="32" t="s">
         <v>17</v>
       </c>
-      <c r="I15" s="33">
+      <c r="I15" s="33" t="e">
         <f>I14+I13</f>
-        <v>0</v>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="16" spans="2:14" x14ac:dyDescent="0.2">
@@ -2319,10 +2321,10 @@
       </c>
     </row>
     <row r="20" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="B20" s="59" t="s">
+      <c r="B20" s="56" t="s">
         <v>24</v>
       </c>
-      <c r="C20" s="59"/>
+      <c r="C20" s="56"/>
       <c r="D20" s="35" t="e">
         <f>EDATE(I6,1)</f>
         <v>#VALUE!</v>
@@ -2340,52 +2342,52 @@
       </c>
     </row>
     <row r="22" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="B22" s="60" t="s">
+      <c r="B22" s="57" t="s">
         <v>27</v>
       </c>
-      <c r="C22" s="60"/>
-      <c r="D22" s="60"/>
-      <c r="E22" s="60"/>
-      <c r="F22" s="60"/>
-      <c r="G22" s="60"/>
-      <c r="H22" s="60"/>
-      <c r="I22" s="60"/>
+      <c r="C22" s="57"/>
+      <c r="D22" s="57"/>
+      <c r="E22" s="57"/>
+      <c r="F22" s="57"/>
+      <c r="G22" s="57"/>
+      <c r="H22" s="57"/>
+      <c r="I22" s="57"/>
     </row>
     <row r="23" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="B23" s="60" t="s">
+      <c r="B23" s="57" t="s">
         <v>28</v>
       </c>
-      <c r="C23" s="60"/>
-      <c r="D23" s="60"/>
-      <c r="E23" s="60"/>
-      <c r="F23" s="60"/>
-      <c r="G23" s="60"/>
-      <c r="H23" s="60"/>
-      <c r="I23" s="60"/>
+      <c r="C23" s="57"/>
+      <c r="D23" s="57"/>
+      <c r="E23" s="57"/>
+      <c r="F23" s="57"/>
+      <c r="G23" s="57"/>
+      <c r="H23" s="57"/>
+      <c r="I23" s="57"/>
     </row>
     <row r="24" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="B24" s="60" t="s">
+      <c r="B24" s="57" t="s">
         <v>29</v>
       </c>
-      <c r="C24" s="60"/>
-      <c r="D24" s="60"/>
-      <c r="E24" s="60"/>
-      <c r="F24" s="60"/>
-      <c r="G24" s="60"/>
-      <c r="H24" s="60"/>
-      <c r="I24" s="60"/>
+      <c r="C24" s="57"/>
+      <c r="D24" s="57"/>
+      <c r="E24" s="57"/>
+      <c r="F24" s="57"/>
+      <c r="G24" s="57"/>
+      <c r="H24" s="57"/>
+      <c r="I24" s="57"/>
     </row>
     <row r="25" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="B25" s="60" t="s">
+      <c r="B25" s="57" t="s">
         <v>30</v>
       </c>
-      <c r="C25" s="60"/>
-      <c r="D25" s="60"/>
-      <c r="E25" s="60"/>
-      <c r="F25" s="60"/>
-      <c r="G25" s="60"/>
-      <c r="H25" s="60"/>
-      <c r="I25" s="60"/>
+      <c r="C25" s="57"/>
+      <c r="D25" s="57"/>
+      <c r="E25" s="57"/>
+      <c r="F25" s="57"/>
+      <c r="G25" s="57"/>
+      <c r="H25" s="57"/>
+      <c r="I25" s="57"/>
     </row>
     <row r="26" spans="1:20" ht="21" x14ac:dyDescent="0.2">
       <c r="B26" s="36" t="s">
@@ -2432,14 +2434,14 @@
     </row>
     <row r="31" spans="1:20" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A31" s="3"/>
-      <c r="B31" s="57"/>
-      <c r="C31" s="57"/>
-      <c r="D31" s="57"/>
-      <c r="E31" s="57"/>
-      <c r="F31" s="57"/>
-      <c r="G31" s="57"/>
-      <c r="H31" s="57"/>
-      <c r="I31" s="57"/>
+      <c r="B31" s="53"/>
+      <c r="C31" s="53"/>
+      <c r="D31" s="53"/>
+      <c r="E31" s="53"/>
+      <c r="F31" s="53"/>
+      <c r="G31" s="53"/>
+      <c r="H31" s="53"/>
+      <c r="I31" s="53"/>
       <c r="K31" s="3"/>
       <c r="L31" s="3"/>
       <c r="M31" s="3"/>
@@ -2475,13 +2477,13 @@
     <row r="35" spans="1:20" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A35" s="3"/>
       <c r="B35" s="1"/>
-      <c r="C35" s="53"/>
-      <c r="D35" s="53"/>
-      <c r="E35" s="53"/>
-      <c r="F35" s="53"/>
-      <c r="G35" s="53"/>
-      <c r="H35" s="53"/>
-      <c r="I35" s="53"/>
+      <c r="C35" s="54"/>
+      <c r="D35" s="54"/>
+      <c r="E35" s="54"/>
+      <c r="F35" s="54"/>
+      <c r="G35" s="54"/>
+      <c r="H35" s="54"/>
+      <c r="I35" s="54"/>
       <c r="K35" s="3"/>
       <c r="L35" s="3"/>
       <c r="M35" s="3"/>
@@ -2496,12 +2498,12 @@
     <row r="36" spans="1:20" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A36" s="3"/>
       <c r="B36" s="1"/>
-      <c r="C36" s="53"/>
-      <c r="D36" s="53"/>
-      <c r="E36" s="53"/>
-      <c r="F36" s="53"/>
-      <c r="G36" s="53"/>
-      <c r="H36" s="53"/>
+      <c r="C36" s="54"/>
+      <c r="D36" s="54"/>
+      <c r="E36" s="54"/>
+      <c r="F36" s="54"/>
+      <c r="G36" s="54"/>
+      <c r="H36" s="54"/>
       <c r="I36" s="1"/>
       <c r="K36" s="3"/>
       <c r="L36" s="3"/>
@@ -2517,12 +2519,12 @@
     <row r="37" spans="1:20" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A37" s="3"/>
       <c r="B37" s="1"/>
-      <c r="C37" s="53"/>
-      <c r="D37" s="53"/>
-      <c r="E37" s="53"/>
-      <c r="F37" s="53"/>
-      <c r="G37" s="53"/>
-      <c r="H37" s="53"/>
+      <c r="C37" s="54"/>
+      <c r="D37" s="54"/>
+      <c r="E37" s="54"/>
+      <c r="F37" s="54"/>
+      <c r="G37" s="54"/>
+      <c r="H37" s="54"/>
       <c r="I37" s="1"/>
       <c r="K37" s="3"/>
       <c r="L37" s="3"/>
@@ -2550,7 +2552,7 @@
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="3.937007874015748E-2" right="3.937007874015748E-2" top="0.39370078740157483" bottom="0.19685039370078741" header="0.39370078740157483" footer="0"/>
-  <pageSetup paperSize="9" scale="73" orientation="portrait" r:id="rId1"/>
+  <pageSetup paperSize="9" scale="74" orientation="portrait" r:id="rId1"/>
   <headerFooter>
     <oddHeader>&amp;C&amp;G</oddHeader>
     <oddFooter>&amp;C&amp;G</oddFooter>
@@ -2601,19 +2603,19 @@
       </c>
     </row>
     <row r="4" spans="1:14" ht="31" x14ac:dyDescent="0.2">
-      <c r="B4" s="54" t="s">
+      <c r="B4" s="58" t="s">
         <v>33</v>
       </c>
-      <c r="C4" s="54"/>
-      <c r="D4" s="54"/>
-      <c r="E4" s="54"/>
-      <c r="F4" s="54"/>
-      <c r="G4" s="54"/>
-      <c r="H4" s="54"/>
-      <c r="I4" s="54"/>
-      <c r="J4" s="54"/>
-      <c r="K4" s="54"/>
-      <c r="L4" s="54"/>
+      <c r="C4" s="58"/>
+      <c r="D4" s="58"/>
+      <c r="E4" s="58"/>
+      <c r="F4" s="58"/>
+      <c r="G4" s="58"/>
+      <c r="H4" s="58"/>
+      <c r="I4" s="58"/>
+      <c r="J4" s="58"/>
+      <c r="K4" s="58"/>
+      <c r="L4" s="58"/>
       <c r="M4" s="5"/>
       <c r="N4" s="6"/>
     </row>
@@ -2796,26 +2798,26 @@
       </c>
     </row>
     <row r="16" spans="1:14" ht="210.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B16" s="55" t="s">
+      <c r="B16" s="59" t="s">
         <v>34</v>
       </c>
-      <c r="C16" s="55"/>
-      <c r="D16" s="55"/>
-      <c r="E16" s="55"/>
-      <c r="F16" s="55"/>
-      <c r="G16" s="55"/>
-      <c r="H16" s="55"/>
-      <c r="I16" s="55"/>
-      <c r="J16" s="55"/>
-      <c r="K16" s="55"/>
-      <c r="L16" s="55"/>
+      <c r="C16" s="59"/>
+      <c r="D16" s="59"/>
+      <c r="E16" s="59"/>
+      <c r="F16" s="59"/>
+      <c r="G16" s="59"/>
+      <c r="H16" s="59"/>
+      <c r="I16" s="59"/>
+      <c r="J16" s="59"/>
+      <c r="K16" s="59"/>
+      <c r="L16" s="59"/>
     </row>
     <row r="17" spans="1:20" x14ac:dyDescent="0.2">
       <c r="E17" s="1"/>
-      <c r="F17" s="56" t="s">
+      <c r="F17" s="60" t="s">
         <v>35</v>
       </c>
-      <c r="G17" s="56"/>
+      <c r="G17" s="60"/>
       <c r="J17" s="1"/>
     </row>
     <row r="18" spans="1:20" x14ac:dyDescent="0.2">
@@ -2859,14 +2861,14 @@
     </row>
     <row r="21" spans="1:20" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A21" s="38"/>
-      <c r="B21" s="57"/>
-      <c r="C21" s="57"/>
-      <c r="D21" s="57"/>
-      <c r="E21" s="57"/>
-      <c r="F21" s="57"/>
-      <c r="G21" s="57"/>
-      <c r="H21" s="57"/>
-      <c r="I21" s="57"/>
+      <c r="B21" s="53"/>
+      <c r="C21" s="53"/>
+      <c r="D21" s="53"/>
+      <c r="E21" s="53"/>
+      <c r="F21" s="53"/>
+      <c r="G21" s="53"/>
+      <c r="H21" s="53"/>
+      <c r="I21" s="53"/>
       <c r="J21" s="38"/>
       <c r="K21" s="1"/>
       <c r="L21" s="1"/>
@@ -2904,13 +2906,13 @@
     <row r="25" spans="1:20" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A25" s="38"/>
       <c r="B25" s="1"/>
-      <c r="C25" s="53"/>
-      <c r="D25" s="53"/>
-      <c r="E25" s="53"/>
-      <c r="F25" s="53"/>
-      <c r="G25" s="53"/>
-      <c r="H25" s="53"/>
-      <c r="I25" s="53"/>
+      <c r="C25" s="54"/>
+      <c r="D25" s="54"/>
+      <c r="E25" s="54"/>
+      <c r="F25" s="54"/>
+      <c r="G25" s="54"/>
+      <c r="H25" s="54"/>
+      <c r="I25" s="54"/>
       <c r="J25" s="38"/>
       <c r="K25" s="1"/>
       <c r="L25" s="1"/>
@@ -2926,12 +2928,12 @@
     <row r="26" spans="1:20" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A26" s="38"/>
       <c r="B26" s="1"/>
-      <c r="C26" s="53"/>
-      <c r="D26" s="53"/>
-      <c r="E26" s="53"/>
-      <c r="F26" s="53"/>
-      <c r="G26" s="53"/>
-      <c r="H26" s="53"/>
+      <c r="C26" s="54"/>
+      <c r="D26" s="54"/>
+      <c r="E26" s="54"/>
+      <c r="F26" s="54"/>
+      <c r="G26" s="54"/>
+      <c r="H26" s="54"/>
       <c r="I26" s="1"/>
       <c r="J26" s="38"/>
       <c r="K26" s="1"/>
@@ -2948,12 +2950,12 @@
     <row r="27" spans="1:20" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A27" s="38"/>
       <c r="B27" s="1"/>
-      <c r="C27" s="53"/>
-      <c r="D27" s="53"/>
-      <c r="E27" s="53"/>
-      <c r="F27" s="53"/>
-      <c r="G27" s="53"/>
-      <c r="H27" s="53"/>
+      <c r="C27" s="54"/>
+      <c r="D27" s="54"/>
+      <c r="E27" s="54"/>
+      <c r="F27" s="54"/>
+      <c r="G27" s="54"/>
+      <c r="H27" s="54"/>
       <c r="I27" s="1"/>
       <c r="J27" s="38"/>
       <c r="K27" s="1"/>
@@ -2980,7 +2982,7 @@
   <phoneticPr fontId="19" type="noConversion"/>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="3.937007874015748E-2" right="3.937007874015748E-2" top="0.39370078740157483" bottom="0.19685039370078741" header="0.39370078740157483" footer="0"/>
-  <pageSetup paperSize="9" scale="86" orientation="portrait" r:id="rId1"/>
+  <pageSetup paperSize="9" scale="87" orientation="portrait" r:id="rId1"/>
   <headerFooter>
     <oddHeader>&amp;C&amp;G</oddHeader>
     <oddFooter>&amp;C&amp;G</oddFooter>

</xml_diff>

<commit_message>
fix(proposal): per-row price formula + correct depreciation/processing totals
The pricing sheet's column I now carries a Table structured-reference
formula (unit price × qty) in the data-row prototype. Replicate that
formula across every generated row instead of overwriting it with a
precomputed value, so Excel stays the source of truth for the line total.

The depreciation_waste/processing summary rows carried their amount in
the qty column with zero weight in G, so the new I = H×G formula totalled
0. Shift those rows one cell left: blank the length column, put a count of
1 in qty (F), and the meters in G — so the total resolves to price × meters.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BE/mgp-service/app/templates/proposal_template.xlsx
+++ b/BE/mgp-service/app/templates/proposal_template.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10517"/>
   <workbookPr filterPrivacy="1" codeName="ThisWorkbook"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0AFCCE0E-96C9-6744-A775-1C44AB45814B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E59FAB8F-389D-8B4A-90D5-AB3EF93FF74D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="19720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="44">
   <si>
     <t>שורה</t>
   </si>
@@ -56,12 +56,6 @@
   </si>
   <si>
     <t>*משקל בק"ג</t>
-  </si>
-  <si>
-    <t>&gt;% Discount - Construction</t>
-  </si>
-  <si>
-    <t>*סה"כ מחיר כולל פחת אחרי הנחה (₪)</t>
   </si>
   <si>
     <t/>
@@ -197,7 +191,7 @@
     <numFmt numFmtId="164" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="165" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
-  <fonts count="21" x14ac:knownFonts="1">
+  <fonts count="20" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -243,13 +237,6 @@
       <sz val="20"/>
       <color theme="1"/>
       <name val="Heebo"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <color rgb="FF2B2D2F"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <b/>
@@ -422,7 +409,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="61">
+  <cellXfs count="59">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -437,18 +424,12 @@
       <alignment horizontal="left" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1" readingOrder="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1" readingOrder="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" readingOrder="2"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -457,19 +438,19 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" readingOrder="2"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1" readingOrder="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" readingOrder="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" readingOrder="2"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="4" fontId="11" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="10" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -478,25 +459,25 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="4" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="4" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="12" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="11" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
@@ -505,22 +486,22 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="14" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="13" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="9" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="8" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -535,48 +516,48 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" readingOrder="2"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="4" fontId="17" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" readingOrder="2"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="12" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="18" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="12" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="18" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="11" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="17" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="11" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="17" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" readingOrder="2"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -591,7 +572,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" readingOrder="2"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -605,43 +586,7 @@
     <cellStyle name="Comma 2" xfId="1" xr:uid="{8B711F14-12F9-DB46-A59C-2DE7D2614634}"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="46">
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <name val="Heebo"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <name val="Heebo"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
+  <dxfs count="40">
     <dxf>
       <font>
         <b val="0"/>
@@ -1103,82 +1048,6 @@
         <top/>
         <bottom/>
       </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <font>
@@ -1686,48 +1555,44 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{5ACB1EC1-21C6-AF40-A140-308C9117B91F}" name="pricing_table25" displayName="pricing_table25" ref="B10:N11" totalsRowShown="0" headerRowDxfId="45" dataDxfId="43" totalsRowDxfId="41" headerRowBorderDxfId="44" tableBorderDxfId="42" totalsRowBorderDxfId="40">
-  <autoFilter ref="B10:N11" xr:uid="{A700047D-2A12-4A24-87A3-5C54C0CD36D6}"/>
-  <tableColumns count="13">
-    <tableColumn id="1" xr3:uid="{9715C0F5-6C58-0C48-A92D-3904FFEE1286}" name="שורה" dataDxfId="39"/>
-    <tableColumn id="2" xr3:uid="{E71665ED-EE05-B544-8402-B3336F34DA2C}" name="מיקום בגג" dataDxfId="38"/>
-    <tableColumn id="3" xr3:uid="{58C96AFC-B01E-D446-8E2A-ACF7B2497559}" name="תאור מוצר" dataDxfId="37"/>
-    <tableColumn id="4" xr3:uid="{D9DC81BB-9F60-0047-86B9-14278D4E2EE7}" name="אורך" dataDxfId="36"/>
-    <tableColumn id="5" xr3:uid="{B9B74024-7469-A149-9639-A328A6F77916}" name="כמות" dataDxfId="35"/>
-    <tableColumn id="6" xr3:uid="{0FF2A4DA-EE5D-564C-892E-1BAF5895A4E7}" name="כמות: ק&quot;ג\יחידות" dataDxfId="34"/>
-    <tableColumn id="7" xr3:uid="{D3D78E52-A52E-C949-9ABD-03AD0269F0BF}" name="מחיר ליחידה (₪)" dataDxfId="33"/>
-    <tableColumn id="8" xr3:uid="{E1EB6162-FB78-1D4F-9435-2CE9366E3552}" name="סה&quot;כ מחיר (₪)" dataDxfId="32">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{5ACB1EC1-21C6-AF40-A140-308C9117B91F}" name="pricing_table25" displayName="pricing_table25" ref="B10:L11" totalsRowShown="0" headerRowDxfId="39" dataDxfId="37" totalsRowDxfId="35" headerRowBorderDxfId="38" tableBorderDxfId="36" totalsRowBorderDxfId="34">
+  <autoFilter ref="B10:L11" xr:uid="{A700047D-2A12-4A24-87A3-5C54C0CD36D6}"/>
+  <tableColumns count="11">
+    <tableColumn id="1" xr3:uid="{9715C0F5-6C58-0C48-A92D-3904FFEE1286}" name="שורה" dataDxfId="33"/>
+    <tableColumn id="2" xr3:uid="{E71665ED-EE05-B544-8402-B3336F34DA2C}" name="מיקום בגג" dataDxfId="32"/>
+    <tableColumn id="3" xr3:uid="{58C96AFC-B01E-D446-8E2A-ACF7B2497559}" name="תאור מוצר" dataDxfId="31"/>
+    <tableColumn id="4" xr3:uid="{D9DC81BB-9F60-0047-86B9-14278D4E2EE7}" name="אורך" dataDxfId="30"/>
+    <tableColumn id="5" xr3:uid="{B9B74024-7469-A149-9639-A328A6F77916}" name="כמות" dataDxfId="29"/>
+    <tableColumn id="6" xr3:uid="{0FF2A4DA-EE5D-564C-892E-1BAF5895A4E7}" name="כמות: ק&quot;ג\יחידות" dataDxfId="28"/>
+    <tableColumn id="7" xr3:uid="{D3D78E52-A52E-C949-9ABD-03AD0269F0BF}" name="מחיר ליחידה (₪)" dataDxfId="27"/>
+    <tableColumn id="8" xr3:uid="{E1EB6162-FB78-1D4F-9435-2CE9366E3552}" name="סה&quot;כ מחיר (₪)" dataDxfId="26">
       <calculatedColumnFormula>pricing_table25[[#This Row],[מחיר ליחידה (₪)]]*pricing_table25[[#This Row],[כמות: ק"ג\יחידות]]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{EAED02B8-7E3B-9B47-8C95-FD7B3D6B7DA0}" name="*כמות פחת" dataDxfId="31" totalsRowDxfId="30"/>
-    <tableColumn id="10" xr3:uid="{8DD3D515-E5F7-3F44-AEEC-EBD82CE3FE68}" name="סה&quot;כ מחיר כולל פחת (₪)" dataDxfId="29" totalsRowDxfId="28"/>
-    <tableColumn id="11" xr3:uid="{B17131E0-AD15-314F-8745-C01B5B56C8B5}" name="*משקל בק&quot;ג" dataDxfId="27" totalsRowDxfId="26"/>
-    <tableColumn id="12" xr3:uid="{8383AEF5-4B81-5944-B8C1-7A02610AD799}" name="&gt;% Discount - Construction" dataDxfId="25" totalsRowDxfId="24"/>
-    <tableColumn id="13" xr3:uid="{A6FF8C60-F61C-014D-BE3D-D97E0E91917D}" name="*סה&quot;כ מחיר כולל פחת אחרי הנחה (₪)" dataDxfId="23" totalsRowDxfId="22"/>
+    <tableColumn id="9" xr3:uid="{EAED02B8-7E3B-9B47-8C95-FD7B3D6B7DA0}" name="*כמות פחת" dataDxfId="25" totalsRowDxfId="24"/>
+    <tableColumn id="10" xr3:uid="{8DD3D515-E5F7-3F44-AEEC-EBD82CE3FE68}" name="סה&quot;כ מחיר כולל פחת (₪)" dataDxfId="23" totalsRowDxfId="22"/>
+    <tableColumn id="11" xr3:uid="{B17131E0-AD15-314F-8745-C01B5B56C8B5}" name="*משקל בק&quot;ג" dataDxfId="21" totalsRowDxfId="20"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium15" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{53B791F9-974C-2D45-9198-4628741EC180}" name="pricing_table34" displayName="pricing_table34" ref="B10:N11" totalsRowShown="0" headerRowDxfId="21" dataDxfId="19" totalsRowDxfId="17" headerRowBorderDxfId="20" tableBorderDxfId="18" totalsRowBorderDxfId="16">
-  <autoFilter ref="B10:N11" xr:uid="{A700047D-2A12-4A24-87A3-5C54C0CD36D6}"/>
-  <tableColumns count="13">
-    <tableColumn id="1" xr3:uid="{C9E84F90-D937-9240-8769-8F47365B79B5}" name="שורה" dataDxfId="15"/>
-    <tableColumn id="2" xr3:uid="{584DEAFB-76D6-C647-A742-316CAAE5BC89}" name="מיקום בגג" dataDxfId="14"/>
-    <tableColumn id="3" xr3:uid="{199A858B-5154-3C42-B14B-B655372B7E72}" name="תאור מוצר" dataDxfId="13"/>
-    <tableColumn id="4" xr3:uid="{044A01A8-0D84-EB4C-A2F1-510AF1F79EC1}" name="אורך" dataDxfId="12"/>
-    <tableColumn id="5" xr3:uid="{23494D31-1003-EC4A-B3E4-56115FE1DC9B}" name="כמות" dataDxfId="11"/>
-    <tableColumn id="6" xr3:uid="{C3ADA01B-011E-AF49-B8EF-BF51E4952D25}" name="כמות: ק&quot;ג\יחידות" dataDxfId="10"/>
-    <tableColumn id="7" xr3:uid="{A4F8123E-37EB-2544-80EC-813AFA9298EC}" name="מחיר ליחידה (₪)" dataDxfId="9"/>
-    <tableColumn id="8" xr3:uid="{891F3848-661F-3446-A7E0-95642AC543B8}" name="סה&quot;כ מחיר (₪)" dataDxfId="8">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{53B791F9-974C-2D45-9198-4628741EC180}" name="pricing_table34" displayName="pricing_table34" ref="B10:L11" totalsRowShown="0" headerRowDxfId="19" dataDxfId="17" totalsRowDxfId="15" headerRowBorderDxfId="18" tableBorderDxfId="16" totalsRowBorderDxfId="14">
+  <autoFilter ref="B10:L11" xr:uid="{A700047D-2A12-4A24-87A3-5C54C0CD36D6}"/>
+  <tableColumns count="11">
+    <tableColumn id="1" xr3:uid="{C9E84F90-D937-9240-8769-8F47365B79B5}" name="שורה" dataDxfId="13"/>
+    <tableColumn id="2" xr3:uid="{584DEAFB-76D6-C647-A742-316CAAE5BC89}" name="מיקום בגג" dataDxfId="12"/>
+    <tableColumn id="3" xr3:uid="{199A858B-5154-3C42-B14B-B655372B7E72}" name="תאור מוצר" dataDxfId="11"/>
+    <tableColumn id="4" xr3:uid="{044A01A8-0D84-EB4C-A2F1-510AF1F79EC1}" name="אורך" dataDxfId="10"/>
+    <tableColumn id="5" xr3:uid="{23494D31-1003-EC4A-B3E4-56115FE1DC9B}" name="כמות" dataDxfId="9"/>
+    <tableColumn id="6" xr3:uid="{C3ADA01B-011E-AF49-B8EF-BF51E4952D25}" name="כמות: ק&quot;ג\יחידות" dataDxfId="8"/>
+    <tableColumn id="7" xr3:uid="{A4F8123E-37EB-2544-80EC-813AFA9298EC}" name="מחיר ליחידה (₪)" dataDxfId="7"/>
+    <tableColumn id="8" xr3:uid="{891F3848-661F-3446-A7E0-95642AC543B8}" name="סה&quot;כ מחיר (₪)" dataDxfId="6">
       <calculatedColumnFormula>pricing_table34[[#This Row],[מחיר ליחידה (₪)]]*pricing_table34[[#This Row],[כמות: ק"ג\יחידות]]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{A50A1AEB-0486-8F4C-A4F6-1B417D72DF83}" name="*כמות פחת" dataDxfId="7" totalsRowDxfId="6"/>
-    <tableColumn id="10" xr3:uid="{3B89E727-3B11-4A40-B717-5C248FA24D57}" name="סה&quot;כ מחיר כולל פחת (₪)" dataDxfId="5" totalsRowDxfId="4"/>
-    <tableColumn id="11" xr3:uid="{981756E0-FF9F-014E-A803-EA2D248E751E}" name="*משקל בק&quot;ג" dataDxfId="3" totalsRowDxfId="2"/>
-    <tableColumn id="12" xr3:uid="{DAD5CC53-679B-024A-96B0-9223C3E03988}" name="&gt;% Discount - Construction" dataDxfId="1"/>
-    <tableColumn id="13" xr3:uid="{7498AF7D-E4AF-4D4F-A51C-BC365E54108A}" name="*סה&quot;כ מחיר כולל פחת אחרי הנחה (₪)" dataDxfId="0"/>
+    <tableColumn id="9" xr3:uid="{A50A1AEB-0486-8F4C-A4F6-1B417D72DF83}" name="*כמות פחת" dataDxfId="5" totalsRowDxfId="4"/>
+    <tableColumn id="10" xr3:uid="{3B89E727-3B11-4A40-B717-5C248FA24D57}" name="סה&quot;כ מחיר כולל פחת (₪)" dataDxfId="3" totalsRowDxfId="2"/>
+    <tableColumn id="11" xr3:uid="{981756E0-FF9F-014E-A803-EA2D248E751E}" name="*משקל בק&quot;ג" dataDxfId="1" totalsRowDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium15" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2058,7 +1923,7 @@
   <sheetPr codeName="Sheet5">
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:T37"/>
+  <dimension ref="A1:R37"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.1640625" defaultRowHeight="20" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="2.5" style="3" customWidth="1"/>
@@ -2072,354 +1937,331 @@
     <col min="10" max="10" width="8.83203125" customWidth="1"/>
     <col min="11" max="11" width="25.6640625" style="3" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="16.1640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="28.5" style="3" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="35.83203125" style="3" bestFit="1" customWidth="1"/>
-    <col min="15" max="16384" width="9.1640625" style="3"/>
+    <col min="13" max="16384" width="9.1640625" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:14" x14ac:dyDescent="0.2">
+    <row r="1" spans="2:12" x14ac:dyDescent="0.2">
       <c r="B1" s="1" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="2" spans="2:14" x14ac:dyDescent="0.2">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="2:12" x14ac:dyDescent="0.2">
       <c r="B2" s="1" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="3" spans="2:14" x14ac:dyDescent="0.2">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="3" spans="2:12" x14ac:dyDescent="0.2">
       <c r="B3" s="1" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="4" spans="2:14" ht="31" x14ac:dyDescent="0.2">
-      <c r="B4" s="55" t="s">
-        <v>9</v>
-      </c>
-      <c r="C4" s="55"/>
-      <c r="D4" s="55"/>
-      <c r="E4" s="55"/>
-      <c r="F4" s="55"/>
-      <c r="G4" s="55"/>
-      <c r="H4" s="55"/>
-      <c r="I4" s="55"/>
+        <v>6</v>
+      </c>
+    </row>
+    <row r="4" spans="2:12" ht="31" x14ac:dyDescent="0.2">
+      <c r="B4" s="53" t="s">
+        <v>7</v>
+      </c>
+      <c r="C4" s="53"/>
+      <c r="D4" s="53"/>
+      <c r="E4" s="53"/>
+      <c r="F4" s="53"/>
+      <c r="G4" s="53"/>
+      <c r="H4" s="53"/>
+      <c r="I4" s="53"/>
       <c r="K4" s="4"/>
       <c r="L4" s="4"/>
-      <c r="M4" s="5"/>
-      <c r="N4" s="6"/>
-    </row>
-    <row r="5" spans="2:14" ht="23" x14ac:dyDescent="0.2">
-      <c r="B5" s="7"/>
-      <c r="C5" s="7"/>
-      <c r="D5" s="7"/>
-      <c r="E5" s="7"/>
-      <c r="F5" s="7"/>
-      <c r="G5" s="7"/>
-      <c r="H5" s="7"/>
-      <c r="I5" s="7"/>
+    </row>
+    <row r="5" spans="2:12" ht="23" x14ac:dyDescent="0.2">
+      <c r="B5" s="5"/>
+      <c r="C5" s="5"/>
+      <c r="D5" s="5"/>
+      <c r="E5" s="5"/>
+      <c r="F5" s="5"/>
+      <c r="G5" s="5"/>
+      <c r="H5" s="5"/>
+      <c r="I5" s="5"/>
       <c r="K5" s="4"/>
       <c r="L5" s="4"/>
-      <c r="M5" s="5"/>
-      <c r="N5" s="6"/>
-    </row>
-    <row r="6" spans="2:14" ht="42" x14ac:dyDescent="0.2">
-      <c r="B6" s="8" t="s">
+    </row>
+    <row r="6" spans="2:12" ht="42" x14ac:dyDescent="0.2">
+      <c r="B6" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="C6" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="H6" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="I6" s="7" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="7" spans="2:12" ht="42" x14ac:dyDescent="0.2">
+      <c r="B7" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="C6" s="9" t="s">
-        <v>36</v>
-      </c>
-      <c r="H6" s="10" t="s">
-        <v>11</v>
-      </c>
-      <c r="I6" s="9" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="7" spans="2:14" ht="42" x14ac:dyDescent="0.2">
-      <c r="B7" s="11" t="s">
-        <v>12</v>
-      </c>
-      <c r="C7" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="H7" s="12"/>
-      <c r="I7" s="9"/>
-    </row>
-    <row r="8" spans="2:14" ht="23" x14ac:dyDescent="0.2">
-      <c r="B8" s="13"/>
-      <c r="C8" s="13"/>
-      <c r="D8" s="13"/>
-      <c r="E8" s="13"/>
-      <c r="F8" s="13"/>
-      <c r="G8" s="13"/>
-      <c r="H8" s="13"/>
-      <c r="I8" s="13"/>
+      <c r="C7" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="H7" s="10"/>
+      <c r="I7" s="7"/>
+    </row>
+    <row r="8" spans="2:12" ht="23" x14ac:dyDescent="0.2">
+      <c r="B8" s="11"/>
+      <c r="C8" s="11"/>
+      <c r="D8" s="11"/>
+      <c r="E8" s="11"/>
+      <c r="F8" s="11"/>
+      <c r="G8" s="11"/>
+      <c r="H8" s="11"/>
+      <c r="I8" s="11"/>
       <c r="K8" s="4"/>
       <c r="L8" s="4"/>
-      <c r="M8" s="5"/>
-      <c r="N8" s="6"/>
-    </row>
-    <row r="9" spans="2:14" ht="3.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="C9" s="14"/>
+    </row>
+    <row r="9" spans="2:12" ht="3.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="C9" s="12"/>
       <c r="K9" s="4"/>
       <c r="L9" s="4"/>
-      <c r="M9" s="6"/>
-      <c r="N9" s="6"/>
-    </row>
-    <row r="10" spans="2:14" s="18" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B10" s="15" t="s">
+    </row>
+    <row r="10" spans="2:12" s="16" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B10" s="13" t="s">
         <v>0</v>
       </c>
-      <c r="C10" s="15" t="s">
+      <c r="C10" s="13" t="s">
+        <v>11</v>
+      </c>
+      <c r="D10" s="13" t="s">
+        <v>12</v>
+      </c>
+      <c r="E10" s="14" t="s">
+        <v>1</v>
+      </c>
+      <c r="F10" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="G10" s="13" t="s">
         <v>13</v>
       </c>
-      <c r="D10" s="15" t="s">
+      <c r="H10" s="13" t="s">
         <v>14</v>
       </c>
-      <c r="E10" s="16" t="s">
-        <v>1</v>
-      </c>
-      <c r="F10" s="15" t="s">
-        <v>2</v>
-      </c>
-      <c r="G10" s="15" t="s">
+      <c r="I10" s="13" t="s">
         <v>15</v>
       </c>
-      <c r="H10" s="15" t="s">
+      <c r="J10" s="15" t="s">
+        <v>3</v>
+      </c>
+      <c r="K10" s="15" t="s">
         <v>16</v>
       </c>
-      <c r="I10" s="15" t="s">
+      <c r="L10" s="15" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="11" spans="2:12" ht="17" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B11" s="44" t="s">
+        <v>37</v>
+      </c>
+      <c r="C11" s="17" t="s">
+        <v>5</v>
+      </c>
+      <c r="D11" s="17"/>
+      <c r="E11" s="18"/>
+      <c r="F11" s="17"/>
+      <c r="G11" s="18"/>
+      <c r="H11" s="18"/>
+      <c r="I11" s="18">
+        <f>pricing_table25[[#This Row],[מחיר ליחידה (₪)]]*pricing_table25[[#This Row],[כמות: ק"ג\יחידות]]</f>
+        <v>0</v>
+      </c>
+      <c r="J11" s="19"/>
+      <c r="K11" s="20"/>
+      <c r="L11" s="20"/>
+    </row>
+    <row r="12" spans="2:12" x14ac:dyDescent="0.2">
+      <c r="H12" s="22" t="s">
         <v>17</v>
       </c>
-      <c r="J10" s="17" t="s">
-        <v>3</v>
-      </c>
-      <c r="K10" s="17" t="s">
-        <v>18</v>
-      </c>
-      <c r="L10" s="17" t="s">
-        <v>4</v>
-      </c>
-      <c r="M10" s="17" t="s">
-        <v>5</v>
-      </c>
-      <c r="N10" s="17" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="11" spans="2:14" ht="17" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B11" s="46" t="s">
-        <v>39</v>
-      </c>
-      <c r="C11" s="19" t="s">
-        <v>7</v>
-      </c>
-      <c r="D11" s="19"/>
-      <c r="E11" s="20"/>
-      <c r="F11" s="19"/>
-      <c r="G11" s="20"/>
-      <c r="H11" s="20"/>
-      <c r="I11" s="20"/>
-      <c r="J11" s="21"/>
-      <c r="K11" s="22"/>
-      <c r="L11" s="22"/>
-      <c r="M11" s="22"/>
-      <c r="N11" s="22"/>
-    </row>
-    <row r="12" spans="2:14" x14ac:dyDescent="0.2">
-      <c r="H12" s="24" t="s">
-        <v>19</v>
-      </c>
-      <c r="I12" s="25">
+      <c r="I12" s="23">
         <f>SUM(I11:I11)</f>
         <v>0</v>
       </c>
-      <c r="J12" s="26">
+      <c r="J12" s="24">
         <f>SUM(J11:J11)</f>
         <v>0</v>
       </c>
-      <c r="K12" s="27" t="s">
-        <v>20</v>
-      </c>
-      <c r="L12" s="28">
+      <c r="K12" s="25" t="s">
+        <v>18</v>
+      </c>
+      <c r="L12" s="26">
         <f>SUM(L11:L11)</f>
         <v>0</v>
       </c>
-      <c r="M12" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="N12" s="28">
-        <f>SUM(N11:N11)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="13" spans="2:14" x14ac:dyDescent="0.2">
-      <c r="H13" s="24" t="s">
-        <v>21</v>
-      </c>
-      <c r="I13" s="52" t="s">
-        <v>45</v>
-      </c>
-      <c r="J13" s="29"/>
-      <c r="K13" s="27"/>
-      <c r="L13" s="30"/>
-      <c r="N13" s="30"/>
-    </row>
-    <row r="14" spans="2:14" x14ac:dyDescent="0.2">
-      <c r="H14" s="23" t="s">
-        <v>22</v>
-      </c>
-      <c r="I14" s="31" t="e">
+    </row>
+    <row r="13" spans="2:12" x14ac:dyDescent="0.2">
+      <c r="H13" s="22" t="s">
+        <v>19</v>
+      </c>
+      <c r="I13" s="50" t="s">
+        <v>43</v>
+      </c>
+      <c r="J13" s="27"/>
+      <c r="K13" s="25"/>
+      <c r="L13" s="28"/>
+    </row>
+    <row r="14" spans="2:12" x14ac:dyDescent="0.2">
+      <c r="H14" s="21" t="s">
+        <v>20</v>
+      </c>
+      <c r="I14" s="29" t="e">
         <f>I13*18%</f>
         <v>#VALUE!</v>
       </c>
     </row>
-    <row r="15" spans="2:14" x14ac:dyDescent="0.2">
-      <c r="H15" s="32" t="s">
-        <v>17</v>
-      </c>
-      <c r="I15" s="33" t="e">
+    <row r="15" spans="2:12" x14ac:dyDescent="0.2">
+      <c r="H15" s="30" t="s">
+        <v>15</v>
+      </c>
+      <c r="I15" s="31" t="e">
         <f>I14+I13</f>
         <v>#VALUE!</v>
       </c>
     </row>
-    <row r="16" spans="2:14" x14ac:dyDescent="0.2">
-      <c r="H16" s="32" t="s">
-        <v>23</v>
-      </c>
-      <c r="I16" s="33">
+    <row r="16" spans="2:12" x14ac:dyDescent="0.2">
+      <c r="H16" s="30" t="s">
+        <v>21</v>
+      </c>
+      <c r="I16" s="31">
         <f>L12</f>
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:20" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:18" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="1"/>
       <c r="G17" s="3"/>
-      <c r="H17" s="32" t="s">
+      <c r="H17" s="30" t="s">
+        <v>39</v>
+      </c>
+      <c r="I17" s="50" t="s">
         <v>41</v>
       </c>
-      <c r="I17" s="52" t="s">
-        <v>43</v>
-      </c>
       <c r="J17" s="3"/>
     </row>
-    <row r="18" spans="1:20" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:18" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="1"/>
       <c r="G18" s="3"/>
-      <c r="H18" s="32" t="s">
+      <c r="H18" s="30" t="s">
+        <v>40</v>
+      </c>
+      <c r="I18" s="50" t="s">
         <v>42</v>
       </c>
-      <c r="I18" s="52" t="s">
-        <v>44</v>
-      </c>
       <c r="J18" s="3"/>
     </row>
-    <row r="19" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:18" x14ac:dyDescent="0.2">
       <c r="B19" s="1" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="20" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="B20" s="56" t="s">
-        <v>24</v>
-      </c>
-      <c r="C20" s="56"/>
-      <c r="D20" s="35" t="e">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="20" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="B20" s="54" t="s">
+        <v>22</v>
+      </c>
+      <c r="C20" s="54"/>
+      <c r="D20" s="33" t="e">
         <f>EDATE(I6,1)</f>
         <v>#VALUE!</v>
       </c>
       <c r="F20" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="G20" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="21" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="B21" s="32" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="22" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="B22" s="55" t="s">
         <v>25</v>
       </c>
-      <c r="G20" s="1" t="s">
+      <c r="C22" s="55"/>
+      <c r="D22" s="55"/>
+      <c r="E22" s="55"/>
+      <c r="F22" s="55"/>
+      <c r="G22" s="55"/>
+      <c r="H22" s="55"/>
+      <c r="I22" s="55"/>
+    </row>
+    <row r="23" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="B23" s="55" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="21" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="B21" s="34" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="22" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="B22" s="57" t="s">
+      <c r="C23" s="55"/>
+      <c r="D23" s="55"/>
+      <c r="E23" s="55"/>
+      <c r="F23" s="55"/>
+      <c r="G23" s="55"/>
+      <c r="H23" s="55"/>
+      <c r="I23" s="55"/>
+    </row>
+    <row r="24" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="B24" s="55" t="s">
         <v>27</v>
       </c>
-      <c r="C22" s="57"/>
-      <c r="D22" s="57"/>
-      <c r="E22" s="57"/>
-      <c r="F22" s="57"/>
-      <c r="G22" s="57"/>
-      <c r="H22" s="57"/>
-      <c r="I22" s="57"/>
-    </row>
-    <row r="23" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="B23" s="57" t="s">
+      <c r="C24" s="55"/>
+      <c r="D24" s="55"/>
+      <c r="E24" s="55"/>
+      <c r="F24" s="55"/>
+      <c r="G24" s="55"/>
+      <c r="H24" s="55"/>
+      <c r="I24" s="55"/>
+    </row>
+    <row r="25" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="B25" s="55" t="s">
         <v>28</v>
       </c>
-      <c r="C23" s="57"/>
-      <c r="D23" s="57"/>
-      <c r="E23" s="57"/>
-      <c r="F23" s="57"/>
-      <c r="G23" s="57"/>
-      <c r="H23" s="57"/>
-      <c r="I23" s="57"/>
-    </row>
-    <row r="24" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="B24" s="57" t="s">
+      <c r="C25" s="55"/>
+      <c r="D25" s="55"/>
+      <c r="E25" s="55"/>
+      <c r="F25" s="55"/>
+      <c r="G25" s="55"/>
+      <c r="H25" s="55"/>
+      <c r="I25" s="55"/>
+    </row>
+    <row r="26" spans="1:18" ht="21" x14ac:dyDescent="0.2">
+      <c r="B26" s="34" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="27" spans="1:18" ht="21" x14ac:dyDescent="0.2">
+      <c r="B27" s="34" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="28" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="B28" s="32"/>
+      <c r="H28" s="8" t="s">
         <v>29</v>
       </c>
-      <c r="C24" s="57"/>
-      <c r="D24" s="57"/>
-      <c r="E24" s="57"/>
-      <c r="F24" s="57"/>
-      <c r="G24" s="57"/>
-      <c r="H24" s="57"/>
-      <c r="I24" s="57"/>
-    </row>
-    <row r="25" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="B25" s="57" t="s">
+    </row>
+    <row r="29" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="B29" s="35"/>
+      <c r="H29" s="8" t="s">
         <v>30</v>
       </c>
-      <c r="C25" s="57"/>
-      <c r="D25" s="57"/>
-      <c r="E25" s="57"/>
-      <c r="F25" s="57"/>
-      <c r="G25" s="57"/>
-      <c r="H25" s="57"/>
-      <c r="I25" s="57"/>
-    </row>
-    <row r="26" spans="1:20" ht="21" x14ac:dyDescent="0.2">
-      <c r="B26" s="36" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="27" spans="1:20" ht="21" x14ac:dyDescent="0.2">
-      <c r="B27" s="36" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="28" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="B28" s="34"/>
-      <c r="H28" s="10" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="29" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="B29" s="37"/>
-      <c r="H29" s="10" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="30" spans="1:20" customFormat="1" ht="74.25" customHeight="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="30" spans="1:18" customFormat="1" ht="74.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="3"/>
-      <c r="B30" s="37"/>
+      <c r="B30" s="35"/>
       <c r="C30" s="1"/>
       <c r="D30" s="1"/>
       <c r="E30" s="2"/>
       <c r="F30" s="1"/>
       <c r="G30" s="1"/>
-      <c r="H30" s="10"/>
+      <c r="H30" s="8"/>
       <c r="I30" s="1"/>
       <c r="K30" s="3"/>
       <c r="L30" s="3"/>
@@ -2429,19 +2271,17 @@
       <c r="P30" s="3"/>
       <c r="Q30" s="3"/>
       <c r="R30" s="3"/>
-      <c r="S30" s="3"/>
-      <c r="T30" s="3"/>
-    </row>
-    <row r="31" spans="1:20" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    </row>
+    <row r="31" spans="1:18" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A31" s="3"/>
-      <c r="B31" s="53"/>
-      <c r="C31" s="53"/>
-      <c r="D31" s="53"/>
-      <c r="E31" s="53"/>
-      <c r="F31" s="53"/>
-      <c r="G31" s="53"/>
-      <c r="H31" s="53"/>
-      <c r="I31" s="53"/>
+      <c r="B31" s="51"/>
+      <c r="C31" s="51"/>
+      <c r="D31" s="51"/>
+      <c r="E31" s="51"/>
+      <c r="F31" s="51"/>
+      <c r="G31" s="51"/>
+      <c r="H31" s="51"/>
+      <c r="I31" s="51"/>
       <c r="K31" s="3"/>
       <c r="L31" s="3"/>
       <c r="M31" s="3"/>
@@ -2450,18 +2290,16 @@
       <c r="P31" s="3"/>
       <c r="Q31" s="3"/>
       <c r="R31" s="3"/>
-      <c r="S31" s="3"/>
-      <c r="T31" s="3"/>
-    </row>
-    <row r="32" spans="1:20" customFormat="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="32" spans="1:18" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A32" s="3"/>
-      <c r="B32" s="37"/>
+      <c r="B32" s="35"/>
       <c r="C32" s="1"/>
       <c r="D32" s="1"/>
       <c r="E32" s="2"/>
       <c r="F32" s="1"/>
       <c r="G32" s="1"/>
-      <c r="H32" s="10"/>
+      <c r="H32" s="8"/>
       <c r="I32" s="1"/>
       <c r="K32" s="3"/>
       <c r="L32" s="3"/>
@@ -2471,19 +2309,17 @@
       <c r="P32" s="3"/>
       <c r="Q32" s="3"/>
       <c r="R32" s="3"/>
-      <c r="S32" s="3"/>
-      <c r="T32" s="3"/>
-    </row>
-    <row r="35" spans="1:20" customFormat="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="35" spans="1:18" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A35" s="3"/>
       <c r="B35" s="1"/>
-      <c r="C35" s="54"/>
-      <c r="D35" s="54"/>
-      <c r="E35" s="54"/>
-      <c r="F35" s="54"/>
-      <c r="G35" s="54"/>
-      <c r="H35" s="54"/>
-      <c r="I35" s="54"/>
+      <c r="C35" s="52"/>
+      <c r="D35" s="52"/>
+      <c r="E35" s="52"/>
+      <c r="F35" s="52"/>
+      <c r="G35" s="52"/>
+      <c r="H35" s="52"/>
+      <c r="I35" s="52"/>
       <c r="K35" s="3"/>
       <c r="L35" s="3"/>
       <c r="M35" s="3"/>
@@ -2492,18 +2328,16 @@
       <c r="P35" s="3"/>
       <c r="Q35" s="3"/>
       <c r="R35" s="3"/>
-      <c r="S35" s="3"/>
-      <c r="T35" s="3"/>
-    </row>
-    <row r="36" spans="1:20" customFormat="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="36" spans="1:18" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A36" s="3"/>
       <c r="B36" s="1"/>
-      <c r="C36" s="54"/>
-      <c r="D36" s="54"/>
-      <c r="E36" s="54"/>
-      <c r="F36" s="54"/>
-      <c r="G36" s="54"/>
-      <c r="H36" s="54"/>
+      <c r="C36" s="52"/>
+      <c r="D36" s="52"/>
+      <c r="E36" s="52"/>
+      <c r="F36" s="52"/>
+      <c r="G36" s="52"/>
+      <c r="H36" s="52"/>
       <c r="I36" s="1"/>
       <c r="K36" s="3"/>
       <c r="L36" s="3"/>
@@ -2513,18 +2347,16 @@
       <c r="P36" s="3"/>
       <c r="Q36" s="3"/>
       <c r="R36" s="3"/>
-      <c r="S36" s="3"/>
-      <c r="T36" s="3"/>
-    </row>
-    <row r="37" spans="1:20" customFormat="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="37" spans="1:18" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A37" s="3"/>
       <c r="B37" s="1"/>
-      <c r="C37" s="54"/>
-      <c r="D37" s="54"/>
-      <c r="E37" s="54"/>
-      <c r="F37" s="54"/>
-      <c r="G37" s="54"/>
-      <c r="H37" s="54"/>
+      <c r="C37" s="52"/>
+      <c r="D37" s="52"/>
+      <c r="E37" s="52"/>
+      <c r="F37" s="52"/>
+      <c r="G37" s="52"/>
+      <c r="H37" s="52"/>
       <c r="I37" s="1"/>
       <c r="K37" s="3"/>
       <c r="L37" s="3"/>
@@ -2534,8 +2366,6 @@
       <c r="P37" s="3"/>
       <c r="Q37" s="3"/>
       <c r="R37" s="3"/>
-      <c r="S37" s="3"/>
-      <c r="T37" s="3"/>
     </row>
   </sheetData>
   <mergeCells count="10">
@@ -2569,7 +2399,7 @@
   <sheetPr codeName="Sheet9">
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:T27"/>
+  <dimension ref="A1:R27"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.1640625" defaultRowHeight="20" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="2.5" style="1" customWidth="1"/>
@@ -2581,273 +2411,257 @@
     <col min="7" max="7" width="20.83203125" style="1" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="15.83203125" style="1" hidden="1" customWidth="1"/>
     <col min="9" max="9" width="15" style="1" hidden="1" customWidth="1"/>
-    <col min="10" max="10" width="8.83203125" style="38" hidden="1" customWidth="1"/>
+    <col min="10" max="10" width="8.83203125" style="36" hidden="1" customWidth="1"/>
     <col min="11" max="11" width="0" style="1" hidden="1" customWidth="1"/>
     <col min="12" max="12" width="15.83203125" style="1" bestFit="1" customWidth="1"/>
     <col min="13" max="16384" width="9.1640625" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.35">
       <c r="B1" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="B2" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="B3" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" ht="31" x14ac:dyDescent="0.2">
+      <c r="B4" s="56" t="s">
+        <v>31</v>
+      </c>
+      <c r="C4" s="56"/>
+      <c r="D4" s="56"/>
+      <c r="E4" s="56"/>
+      <c r="F4" s="56"/>
+      <c r="G4" s="56"/>
+      <c r="H4" s="56"/>
+      <c r="I4" s="56"/>
+      <c r="J4" s="56"/>
+      <c r="K4" s="56"/>
+      <c r="L4" s="56"/>
+    </row>
+    <row r="5" spans="1:12" ht="23" x14ac:dyDescent="0.35">
+      <c r="B5" s="5"/>
+      <c r="C5" s="5"/>
+      <c r="D5" s="5"/>
+      <c r="E5" s="5"/>
+      <c r="F5" s="5"/>
+      <c r="G5" s="5"/>
+      <c r="H5" s="11"/>
+      <c r="I5" s="11"/>
+      <c r="K5" s="37"/>
+      <c r="L5" s="37"/>
+    </row>
+    <row r="6" spans="1:12" ht="42" x14ac:dyDescent="0.35">
+      <c r="B6" s="6" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="B2" s="1" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="B3" s="1" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="4" spans="1:14" ht="31" x14ac:dyDescent="0.2">
-      <c r="B4" s="58" t="s">
-        <v>33</v>
-      </c>
-      <c r="C4" s="58"/>
-      <c r="D4" s="58"/>
-      <c r="E4" s="58"/>
-      <c r="F4" s="58"/>
-      <c r="G4" s="58"/>
-      <c r="H4" s="58"/>
-      <c r="I4" s="58"/>
-      <c r="J4" s="58"/>
-      <c r="K4" s="58"/>
-      <c r="L4" s="58"/>
-      <c r="M4" s="5"/>
-      <c r="N4" s="6"/>
-    </row>
-    <row r="5" spans="1:14" ht="23" x14ac:dyDescent="0.35">
-      <c r="B5" s="7"/>
-      <c r="C5" s="7"/>
-      <c r="D5" s="7"/>
-      <c r="E5" s="7"/>
-      <c r="F5" s="7"/>
-      <c r="G5" s="7"/>
-      <c r="H5" s="13"/>
-      <c r="I5" s="13"/>
-      <c r="K5" s="39"/>
-      <c r="L5" s="39"/>
-      <c r="M5" s="5"/>
-      <c r="N5" s="6"/>
-    </row>
-    <row r="6" spans="1:14" ht="42" x14ac:dyDescent="0.35">
-      <c r="B6" s="8" t="s">
+      <c r="C6" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="F6" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="G6" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="H6" s="36"/>
+      <c r="J6" s="1"/>
+    </row>
+    <row r="7" spans="1:12" ht="42" x14ac:dyDescent="0.35">
+      <c r="B7" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="C6" s="9" t="s">
-        <v>36</v>
-      </c>
-      <c r="F6" s="10" t="s">
+      <c r="C7" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="F7" s="10"/>
+      <c r="G7" s="7"/>
+      <c r="H7" s="36"/>
+      <c r="J7" s="1"/>
+    </row>
+    <row r="8" spans="1:12" ht="23" x14ac:dyDescent="0.35">
+      <c r="B8" s="11"/>
+      <c r="C8" s="11"/>
+      <c r="D8" s="11"/>
+      <c r="E8" s="11"/>
+      <c r="F8" s="11"/>
+      <c r="G8" s="11"/>
+      <c r="H8" s="11"/>
+      <c r="I8" s="11"/>
+      <c r="K8" s="37"/>
+      <c r="L8" s="37"/>
+    </row>
+    <row r="9" spans="1:12" ht="3.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="C9" s="12"/>
+      <c r="K9" s="37"/>
+      <c r="L9" s="37"/>
+    </row>
+    <row r="10" spans="1:12" s="16" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A10" s="38"/>
+      <c r="B10" s="13" t="s">
+        <v>0</v>
+      </c>
+      <c r="C10" s="13" t="s">
         <v>11</v>
       </c>
-      <c r="G6" s="9" t="s">
+      <c r="D10" s="13" t="s">
+        <v>12</v>
+      </c>
+      <c r="E10" s="14" t="s">
+        <v>1</v>
+      </c>
+      <c r="F10" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="G10" s="13" t="s">
+        <v>13</v>
+      </c>
+      <c r="H10" s="13" t="s">
+        <v>14</v>
+      </c>
+      <c r="I10" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="J10" s="39" t="s">
+        <v>3</v>
+      </c>
+      <c r="K10" s="39" t="s">
+        <v>16</v>
+      </c>
+      <c r="L10" s="39" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" ht="17" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B11" s="44" t="s">
         <v>38</v>
       </c>
-      <c r="H6" s="38"/>
-      <c r="J6" s="1"/>
-    </row>
-    <row r="7" spans="1:14" ht="42" x14ac:dyDescent="0.35">
-      <c r="B7" s="11" t="s">
-        <v>12</v>
-      </c>
-      <c r="C7" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="F7" s="12"/>
-      <c r="G7" s="9"/>
-      <c r="H7" s="38"/>
-      <c r="J7" s="1"/>
-    </row>
-    <row r="8" spans="1:14" ht="23" x14ac:dyDescent="0.35">
-      <c r="B8" s="13"/>
-      <c r="C8" s="13"/>
-      <c r="D8" s="13"/>
-      <c r="E8" s="13"/>
-      <c r="F8" s="13"/>
-      <c r="G8" s="13"/>
-      <c r="H8" s="13"/>
-      <c r="I8" s="13"/>
-      <c r="K8" s="39"/>
-      <c r="L8" s="39"/>
-      <c r="M8" s="5"/>
-      <c r="N8" s="6"/>
-    </row>
-    <row r="9" spans="1:14" ht="3.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="C9" s="14"/>
-      <c r="K9" s="39"/>
-      <c r="L9" s="39"/>
-      <c r="M9" s="6"/>
-      <c r="N9" s="6"/>
-    </row>
-    <row r="10" spans="1:14" s="18" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="40"/>
-      <c r="B10" s="15" t="s">
-        <v>0</v>
-      </c>
-      <c r="C10" s="15" t="s">
-        <v>13</v>
-      </c>
-      <c r="D10" s="15" t="s">
-        <v>14</v>
-      </c>
-      <c r="E10" s="16" t="s">
-        <v>1</v>
-      </c>
-      <c r="F10" s="15" t="s">
-        <v>2</v>
-      </c>
-      <c r="G10" s="15" t="s">
-        <v>15</v>
-      </c>
-      <c r="H10" s="15" t="s">
-        <v>16</v>
-      </c>
-      <c r="I10" s="15" t="s">
+      <c r="C11" s="17"/>
+      <c r="D11" s="17"/>
+      <c r="E11" s="18"/>
+      <c r="F11" s="17"/>
+      <c r="G11" s="18"/>
+      <c r="H11" s="18"/>
+      <c r="I11" s="18"/>
+      <c r="J11" s="18"/>
+      <c r="K11" s="40"/>
+      <c r="L11" s="41"/>
+    </row>
+    <row r="12" spans="1:12" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="G12" s="45" t="s">
+        <v>21</v>
+      </c>
+      <c r="H12" s="46" t="s">
         <v>17</v>
       </c>
-      <c r="J10" s="41" t="s">
-        <v>3</v>
-      </c>
-      <c r="K10" s="41" t="s">
-        <v>18</v>
-      </c>
-      <c r="L10" s="41" t="s">
-        <v>4</v>
-      </c>
-      <c r="M10" s="17" t="s">
-        <v>5</v>
-      </c>
-      <c r="N10" s="17" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="11" spans="1:14" ht="17" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B11" s="46" t="s">
-        <v>40</v>
-      </c>
-      <c r="C11" s="19"/>
-      <c r="D11" s="19"/>
-      <c r="E11" s="20"/>
-      <c r="F11" s="19"/>
-      <c r="G11" s="20"/>
-      <c r="H11" s="20"/>
-      <c r="I11" s="20"/>
-      <c r="J11" s="20"/>
-      <c r="K11" s="42"/>
-      <c r="L11" s="43"/>
-      <c r="M11" s="43"/>
-      <c r="N11" s="43"/>
-    </row>
-    <row r="12" spans="1:14" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="G12" s="47" t="s">
-        <v>23</v>
-      </c>
-      <c r="H12" s="48" t="s">
-        <v>19</v>
-      </c>
-      <c r="I12" s="49">
+      <c r="I12" s="47">
         <f>SUM(I11:I11)</f>
         <v>0</v>
       </c>
-      <c r="J12" s="49">
+      <c r="J12" s="47">
         <f>SUM(J11:J11)</f>
         <v>0</v>
       </c>
-      <c r="K12" s="44" t="s">
-        <v>20</v>
-      </c>
-      <c r="L12" s="50">
+      <c r="K12" s="42" t="s">
+        <v>18</v>
+      </c>
+      <c r="L12" s="48">
         <f>SUM(L11:L11)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:14" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="G13" s="32" t="s">
+    <row r="13" spans="1:12" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="G13" s="30" t="s">
+        <v>39</v>
+      </c>
+      <c r="H13" s="30"/>
+      <c r="I13" s="49"/>
+      <c r="J13" s="49"/>
+      <c r="K13" s="30"/>
+      <c r="L13" s="50" t="s">
         <v>41</v>
       </c>
-      <c r="H13" s="32"/>
-      <c r="I13" s="51"/>
-      <c r="J13" s="51"/>
-      <c r="K13" s="32"/>
-      <c r="L13" s="52" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="14" spans="1:14" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="G14" s="32" t="s">
+    </row>
+    <row r="14" spans="1:12" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="G14" s="30" t="s">
+        <v>40</v>
+      </c>
+      <c r="H14" s="30"/>
+      <c r="I14" s="49"/>
+      <c r="J14" s="49"/>
+      <c r="K14" s="30"/>
+      <c r="L14" s="50" t="s">
         <v>42</v>
       </c>
-      <c r="H14" s="32"/>
-      <c r="I14" s="51"/>
-      <c r="J14" s="51"/>
-      <c r="K14" s="32"/>
-      <c r="L14" s="52" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="15" spans="1:14" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="H15" s="23" t="s">
-        <v>22</v>
-      </c>
-      <c r="I15" s="31">
+    </row>
+    <row r="15" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="H15" s="21" t="s">
+        <v>20</v>
+      </c>
+      <c r="I15" s="29">
         <f>I12*18%</f>
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:14" ht="210.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B16" s="59" t="s">
-        <v>34</v>
-      </c>
-      <c r="C16" s="59"/>
-      <c r="D16" s="59"/>
-      <c r="E16" s="59"/>
-      <c r="F16" s="59"/>
-      <c r="G16" s="59"/>
-      <c r="H16" s="59"/>
-      <c r="I16" s="59"/>
-      <c r="J16" s="59"/>
-      <c r="K16" s="59"/>
-      <c r="L16" s="59"/>
-    </row>
-    <row r="17" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:12" ht="210.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B16" s="57" t="s">
+        <v>32</v>
+      </c>
+      <c r="C16" s="57"/>
+      <c r="D16" s="57"/>
+      <c r="E16" s="57"/>
+      <c r="F16" s="57"/>
+      <c r="G16" s="57"/>
+      <c r="H16" s="57"/>
+      <c r="I16" s="57"/>
+      <c r="J16" s="57"/>
+      <c r="K16" s="57"/>
+      <c r="L16" s="57"/>
+    </row>
+    <row r="17" spans="1:18" x14ac:dyDescent="0.2">
       <c r="E17" s="1"/>
-      <c r="F17" s="60" t="s">
-        <v>35</v>
-      </c>
-      <c r="G17" s="60"/>
+      <c r="F17" s="58" t="s">
+        <v>33</v>
+      </c>
+      <c r="G17" s="58"/>
       <c r="J17" s="1"/>
     </row>
-    <row r="18" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="B18" s="45"/>
-      <c r="C18" s="45"/>
-      <c r="D18" s="45"/>
-      <c r="E18" s="45"/>
-      <c r="F18" s="10"/>
-      <c r="G18" s="45"/>
-      <c r="H18" s="45"/>
-      <c r="I18" s="45"/>
+    <row r="18" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="B18" s="43"/>
+      <c r="C18" s="43"/>
+      <c r="D18" s="43"/>
+      <c r="E18" s="43"/>
+      <c r="F18" s="8"/>
+      <c r="G18" s="43"/>
+      <c r="H18" s="43"/>
+      <c r="I18" s="43"/>
       <c r="J18" s="1"/>
     </row>
-    <row r="19" spans="1:20" ht="78" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B19" s="37"/>
+    <row r="19" spans="1:18" ht="78" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B19" s="35"/>
       <c r="E19" s="1"/>
-      <c r="F19" s="10"/>
+      <c r="F19" s="8"/>
       <c r="J19" s="1"/>
     </row>
-    <row r="20" spans="1:20" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A20" s="38"/>
-      <c r="B20" s="37"/>
+    <row r="20" spans="1:18" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A20" s="36"/>
+      <c r="B20" s="35"/>
       <c r="C20" s="1"/>
       <c r="D20" s="1"/>
       <c r="E20" s="2"/>
       <c r="F20" s="1"/>
       <c r="G20" s="1"/>
-      <c r="H20" s="10"/>
+      <c r="H20" s="8"/>
       <c r="I20" s="1"/>
-      <c r="J20" s="38"/>
+      <c r="J20" s="36"/>
       <c r="K20" s="1"/>
       <c r="L20" s="1"/>
       <c r="M20" s="3"/>
@@ -2856,20 +2670,18 @@
       <c r="P20" s="3"/>
       <c r="Q20" s="3"/>
       <c r="R20" s="3"/>
-      <c r="S20" s="3"/>
-      <c r="T20" s="3"/>
-    </row>
-    <row r="21" spans="1:20" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A21" s="38"/>
-      <c r="B21" s="53"/>
-      <c r="C21" s="53"/>
-      <c r="D21" s="53"/>
-      <c r="E21" s="53"/>
-      <c r="F21" s="53"/>
-      <c r="G21" s="53"/>
-      <c r="H21" s="53"/>
-      <c r="I21" s="53"/>
-      <c r="J21" s="38"/>
+    </row>
+    <row r="21" spans="1:18" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A21" s="36"/>
+      <c r="B21" s="51"/>
+      <c r="C21" s="51"/>
+      <c r="D21" s="51"/>
+      <c r="E21" s="51"/>
+      <c r="F21" s="51"/>
+      <c r="G21" s="51"/>
+      <c r="H21" s="51"/>
+      <c r="I21" s="51"/>
+      <c r="J21" s="36"/>
       <c r="K21" s="1"/>
       <c r="L21" s="1"/>
       <c r="M21" s="3"/>
@@ -2878,20 +2690,18 @@
       <c r="P21" s="3"/>
       <c r="Q21" s="3"/>
       <c r="R21" s="3"/>
-      <c r="S21" s="3"/>
-      <c r="T21" s="3"/>
-    </row>
-    <row r="22" spans="1:20" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A22" s="38"/>
-      <c r="B22" s="37"/>
+    </row>
+    <row r="22" spans="1:18" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A22" s="36"/>
+      <c r="B22" s="35"/>
       <c r="C22" s="1"/>
       <c r="D22" s="1"/>
       <c r="E22" s="2"/>
       <c r="F22" s="1"/>
       <c r="G22" s="1"/>
-      <c r="H22" s="10"/>
+      <c r="H22" s="8"/>
       <c r="I22" s="1"/>
-      <c r="J22" s="38"/>
+      <c r="J22" s="36"/>
       <c r="K22" s="1"/>
       <c r="L22" s="1"/>
       <c r="M22" s="3"/>
@@ -2900,20 +2710,18 @@
       <c r="P22" s="3"/>
       <c r="Q22" s="3"/>
       <c r="R22" s="3"/>
-      <c r="S22" s="3"/>
-      <c r="T22" s="3"/>
-    </row>
-    <row r="25" spans="1:20" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A25" s="38"/>
+    </row>
+    <row r="25" spans="1:18" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A25" s="36"/>
       <c r="B25" s="1"/>
-      <c r="C25" s="54"/>
-      <c r="D25" s="54"/>
-      <c r="E25" s="54"/>
-      <c r="F25" s="54"/>
-      <c r="G25" s="54"/>
-      <c r="H25" s="54"/>
-      <c r="I25" s="54"/>
-      <c r="J25" s="38"/>
+      <c r="C25" s="52"/>
+      <c r="D25" s="52"/>
+      <c r="E25" s="52"/>
+      <c r="F25" s="52"/>
+      <c r="G25" s="52"/>
+      <c r="H25" s="52"/>
+      <c r="I25" s="52"/>
+      <c r="J25" s="36"/>
       <c r="K25" s="1"/>
       <c r="L25" s="1"/>
       <c r="M25" s="3"/>
@@ -2922,20 +2730,18 @@
       <c r="P25" s="3"/>
       <c r="Q25" s="3"/>
       <c r="R25" s="3"/>
-      <c r="S25" s="3"/>
-      <c r="T25" s="3"/>
-    </row>
-    <row r="26" spans="1:20" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A26" s="38"/>
+    </row>
+    <row r="26" spans="1:18" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A26" s="36"/>
       <c r="B26" s="1"/>
-      <c r="C26" s="54"/>
-      <c r="D26" s="54"/>
-      <c r="E26" s="54"/>
-      <c r="F26" s="54"/>
-      <c r="G26" s="54"/>
-      <c r="H26" s="54"/>
+      <c r="C26" s="52"/>
+      <c r="D26" s="52"/>
+      <c r="E26" s="52"/>
+      <c r="F26" s="52"/>
+      <c r="G26" s="52"/>
+      <c r="H26" s="52"/>
       <c r="I26" s="1"/>
-      <c r="J26" s="38"/>
+      <c r="J26" s="36"/>
       <c r="K26" s="1"/>
       <c r="L26" s="1"/>
       <c r="M26" s="3"/>
@@ -2944,20 +2750,18 @@
       <c r="P26" s="3"/>
       <c r="Q26" s="3"/>
       <c r="R26" s="3"/>
-      <c r="S26" s="3"/>
-      <c r="T26" s="3"/>
-    </row>
-    <row r="27" spans="1:20" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A27" s="38"/>
+    </row>
+    <row r="27" spans="1:18" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A27" s="36"/>
       <c r="B27" s="1"/>
-      <c r="C27" s="54"/>
-      <c r="D27" s="54"/>
-      <c r="E27" s="54"/>
-      <c r="F27" s="54"/>
-      <c r="G27" s="54"/>
-      <c r="H27" s="54"/>
+      <c r="C27" s="52"/>
+      <c r="D27" s="52"/>
+      <c r="E27" s="52"/>
+      <c r="F27" s="52"/>
+      <c r="G27" s="52"/>
+      <c r="H27" s="52"/>
       <c r="I27" s="1"/>
-      <c r="J27" s="38"/>
+      <c r="J27" s="36"/>
       <c r="K27" s="1"/>
       <c r="L27" s="1"/>
       <c r="M27" s="3"/>
@@ -2966,8 +2770,6 @@
       <c r="P27" s="3"/>
       <c r="Q27" s="3"/>
       <c r="R27" s="3"/>
-      <c r="S27" s="3"/>
-      <c r="T27" s="3"/>
     </row>
   </sheetData>
   <mergeCells count="7">
@@ -2979,7 +2781,7 @@
     <mergeCell ref="C25:I25"/>
     <mergeCell ref="C26:H26"/>
   </mergeCells>
-  <phoneticPr fontId="19" type="noConversion"/>
+  <phoneticPr fontId="18" type="noConversion"/>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="3.937007874015748E-2" right="3.937007874015748E-2" top="0.39370078740157483" bottom="0.19685039370078741" header="0.39370078740157483" footer="0"/>
   <pageSetup paperSize="9" scale="87" orientation="portrait" r:id="rId1"/>

</xml_diff>